<commit_message>
Dodaj harmonogram płatności (zaliczka max 40%, 15% przy wniosku końcowym)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Av3yRtjc51k31HhvjViJWB
</commit_message>
<xml_diff>
--- a/Cashflow_SZMO.xlsx
+++ b/Cashflow_SZMO.xlsx
@@ -10,7 +10,8 @@
   <sheets>
     <sheet name="Podsumowanie" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Założenia" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Cashflow" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Harmonogram płatności" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Cashflow" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="167">
   <si>
     <t xml:space="preserve">Cashflow projektu SZMO – podsumowanie</t>
   </si>
@@ -87,6 +88,12 @@
     <t xml:space="preserve">Jeśli &gt; limit pożyczki, potrzebne dodatkowe finansowanie pomostowe</t>
   </si>
   <si>
+    <t xml:space="preserve">Szczyt przejściowego zapotrzebowania na gotówkę – scen. 3 (wg umowy: zaliczka 40% + 15% na koniec)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wariant zgodny z zapisami umowy o dofinansowanie</t>
+  </si>
+  <si>
     <t xml:space="preserve">Niedobór finansowania w wybranym scenariuszu</t>
   </si>
   <si>
@@ -96,6 +103,9 @@
     <t xml:space="preserve">Miesiąc największego zapotrzebowania – scen. 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Miesiąc największego zapotrzebowania – scen. 3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Miesiąc największego zapotrzebowania – scen. 2</t>
   </si>
   <si>
@@ -147,6 +157,9 @@
     <t xml:space="preserve">Smart-ELIT sp. z o.o. · okres realizacji 01.09.2026–31.08.2027 · kolor niebieski = dane wejściowe (z wniosku lub założenie), czarny = formuły</t>
   </si>
   <si>
+    <t xml:space="preserve">Scen. 1: zaliczka na początku kwartału = 85% kosztów kwalif. kolejnych 3 mies. | Scen. 2: refundacja 85% kosztów kwartału z opóźnieniem | Scen. 3: 1. zaliczka = max % z B11, kolejne zaliczki kwartalnie wg potrzeb (niewykorzystana zaliczka ≤ B11, łącznie ≤ 100% − B12), reszta po wniosku końcowym.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stopa dofinansowania</t>
   </si>
   <si>
@@ -177,19 +190,28 @@
     <t xml:space="preserve">ZAŁOŻENIE – zmień, jeśli chcesz utrzymywać rezerwę</t>
   </si>
   <si>
-    <t xml:space="preserve">Scenariusz wpływu dofinansowania (1 = zaliczki, 2 = refundacja)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZAŁOŻENIE – wniosek nie określa trybu wypłaty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opóźnienie wypłaty refundacji po zamknięciu kwartału (mies.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZAŁOŻENIE – dot. scenariusza 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scenariusz 1: zaliczka na początku kwartału (wrz, gru, mar, cze) = 85% kosztów kwalifikowalnych kolejnych 3 mies.  |  Scenariusz 2: refundacja 85% kosztów kwartału z opóźnieniem jak wyżej (ostatnia transza po okresie projektu).</t>
+    <t xml:space="preserve">Scenariusz wpływu dofinansowania (1 / 2 / 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 = zaliczki kwartalne; 2 = refundacja kwartalna; 3 = wg umowy (zaliczka max 40%, 15% przy wniosku końcowym)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opóźnienie wypłaty refundacji / płatności końcowej (mies.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZAŁOŻENIE – dot. scenariuszy 2 i 3 (od końca kwartału / od końca projektu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maksymalna zaliczka (% dofinansowania) – scen. 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UMOWA O DOFINANSOWANIE: zaliczka maks. 40% dofinansowania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Płatność końcowa w formie refundacji (% dofinansowania) – scen. 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UMOWA O DOFINANSOWANIE: 15% wypłacane przy wniosku o płatność końcową</t>
   </si>
   <si>
     <t xml:space="preserve">Zakupy i przychody – harmonogram płatności</t>
@@ -303,6 +325,90 @@
     <t xml:space="preserve">Wynagrodzenia przyjęto jako koszt całkowity pracodawcy („brutto brutto”) i zakładamy wypłatę w miesiącu poniesienia kosztu (podejście ostrożne dla płynności; w praktyce część – ZUS/PIT – płatna do 20. dnia następnego miesiąca).</t>
   </si>
   <si>
+    <t xml:space="preserve">Harmonogram płatności dofinansowania – wg zapisów umowy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaliczka maks. 40% dofinansowania; 15% dofinansowania wypłacane w formie refundacji po wniosku o płatność końcową. Terminy kwartalnych zaliczek i opóźnienie płatności końcowej to założenia (Założenia!B10). Arkusz zawsze pokazuje scenariusz 3, niezależnie od wyboru w Założeniach.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dofinansowanie ogółem (PLN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maksymalna zaliczka (PLN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Płatność końcowa – 15% (PLN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Płatność</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Termin (miesiąc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kwota (PLN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% dofinansowania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Narastająco (PLN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Narastająco %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niewykorzystana zaliczka po wypłacie (PLN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaliczka nr 1 – na start projektu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pierwsza zaliczka w maksymalnej wysokości 40% dofinansowania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaliczka nr 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzupełnienie zaliczki na potrzeby kolejnego kwartału (po rozliczeniu wydatków)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaliczka nr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaliczka nr 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jw.; łącznie zaliczki i płatności pośrednie ≤ 85% dofinansowania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Płatność końcowa (refundacja po wniosku o płatność końcową)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wniosek końcowy po 31.08.2027; wypłata poza okresem realizacji projektu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrola zapisów umowy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suma płatności = dofinansowanie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Najwyższa niewykorzystana zaliczka ≤ 40% dofinansowania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Płatność końcowa ≥ 15% dofinansowania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wypłaty przed wnioskiem końcowym ≤ 85% dofinansowania</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cashflow projektu SZMO – miesięcznie (PLN)</t>
   </si>
   <si>
@@ -394,6 +500,27 @@
   </si>
   <si>
     <t xml:space="preserve">Skumulowany przepływ netto BEZ pożyczki – scen. 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wg umowy (scenariusz 3) – wpływ: zaliczki + płatność końcowa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skumulowany przepływ netto BEZ pożyczki – scen. 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niewykorzystana zaliczka po wypłacie (scen. 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wydatki kwalifikowalne narastająco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wpłaty dofinansowania narastająco (scen. 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niewykorzystana zaliczka na początek miesiąca (scen. 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dofinansowanie ogółem (zaokrąglone)</t>
   </si>
   <si>
     <t xml:space="preserve">Pożyczka właścicielska jest uruchamiana automatycznie tylko do poziomu niedoboru gotówki (do limitu z Założeń); spłata pożyczek wspólnikom nie jest w modelu (brak informacji we wniosku). Kolumna „Po projekcie” to wpływy po 31.08.2027 (np. rozliczenie ostatniej transzy).</t>
@@ -403,7 +530,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;[RED]\(#,##0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="0%;\-0%;\-"/>
@@ -412,6 +539,7 @@
     <numFmt numFmtId="169" formatCode="0"/>
     <numFmt numFmtId="170" formatCode="0.00;\-0.00;\-"/>
     <numFmt numFmtId="171" formatCode="0.00"/>
+    <numFmt numFmtId="172" formatCode="0.0%"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -572,7 +700,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -654,6 +782,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1027,22 +1167,22 @@
                 <c:formatCode>#,##0.00;[RED]\(#,##0.00\);\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>166195.8</c:v>
+                  <c:v>239952.01</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46111</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>153000.97</c:v>
+                  <c:v>79244.76</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>18261.53</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>29103.13</c:v>
+                  <c:v>56952.6</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>145229.13</c:v>
@@ -1054,13 +1194,13 @@
                   <c:v>25628.67</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>135454.13</c:v>
+                  <c:v>56952.6</c:v>
                 </c:pt>
                 <c:pt idx="10">
+                  <c:v>12423.2</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>23903.67</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1068,8 +1208,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25555429"/>
-        <c:axId val="58023075"/>
+        <c:axId val="71421515"/>
+        <c:axId val="69056934"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1178,19 +1318,19 @@
                 <c:formatCode>#,##0.00;[RED]\(#,##0.00\);\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>133393.2</c:v>
+                  <c:v>207149.41</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>55716.1</c:v>
+                  <c:v>129472.31</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>27645.21</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>38691.07</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>84802.07</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>27849.47</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -1205,13 +1345,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>78501.53</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>27298.93</c:v>
+                  <c:v>-38779.4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>-89982</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1226,11 +1366,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="25555429"/>
-        <c:axId val="58023075"/>
+        <c:axId val="71421515"/>
+        <c:axId val="69056934"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="25555429"/>
+        <c:axId val="71421515"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1262,7 +1402,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58023075"/>
+        <c:crossAx val="69056934"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1270,7 +1410,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58023075"/>
+        <c:axId val="69056934"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1312,7 +1452,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25555429"/>
+        <c:crossAx val="71421515"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1370,13 +1510,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>160560</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>2436840</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>48</xdr:row>
       <xdr:rowOff>161640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -1385,7 +1525,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="5715000"/>
+        <a:off x="0" y="6095880"/>
         <a:ext cx="8639640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -1579,7 +1719,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="70"/>
@@ -1686,7 +1826,7 @@
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">MIN(Cashflow!B28:M28)</f>
-        <v>0</v>
+        <v>-89982</v>
       </c>
       <c r="C11" s="2"/>
     </row>
@@ -1719,8 +1859,8 @@
         <v>21</v>
       </c>
       <c r="B14" s="5" t="n">
-        <f aca="false">Cashflow!O29</f>
-        <v>0</v>
+        <f aca="false">-MIN(0,MIN(Cashflow!B38:M38))</f>
+        <v>214728.47</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>22</v>
@@ -1730,94 +1870,76 @@
       <c r="A15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="7" t="str">
+      <c r="B15" s="5" t="n">
+        <f aca="false">Cashflow!O29</f>
+        <v>89982</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="7" t="str">
         <f aca="false">INDEX(Cashflow!B4:M4,MATCH(MIN(Cashflow!B35:M35),Cashflow!B35:M35,0))</f>
         <v>sie 2027</v>
       </c>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="7" t="str">
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="7" t="str">
+        <f aca="false">INDEX(Cashflow!B4:M4,MATCH(MIN(Cashflow!B38:M38),Cashflow!B38:M38,0))</f>
+        <v>sie 2027</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="7" t="str">
         <f aca="false">INDEX(Cashflow!B4:M4,MATCH(MIN(Cashflow!B36:M36),Cashflow!B36:M36,0))</f>
         <v>cze 2027</v>
       </c>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="C18" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="3" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="C21" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="D21" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="5" t="n">
         <f aca="false">Cashflow!O10</f>
         <v>542288</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C22" s="9" t="n">
         <v>542288</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <f aca="false">ROUND(B20-C20,2)</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="8" t="str">
-        <f aca="false">IF(ABS(D20)&lt;=0.05,"OK","SPRAWDŹ")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B21" s="5" t="n">
-        <f aca="false">SUM(Cashflow!B7:M7)+Cashflow!O11</f>
-        <v>244093</v>
-      </c>
-      <c r="C21" s="9" t="n">
-        <v>244093</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <f aca="false">ROUND(B21-C21,2)</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="8" t="str">
-        <f aca="false">IF(ABS(D21)&lt;=0.05,"OK","SPRAWDŹ")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="5" t="n">
-        <f aca="false">SUM(Cashflow!B8:M8)+Cashflow!O12</f>
-        <v>165246.3</v>
-      </c>
-      <c r="C22" s="9" t="n">
-        <v>165246.3</v>
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">ROUND(B22-C22,2)</f>
@@ -1830,14 +1952,14 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" s="5" t="n">
-        <f aca="false">SUM(Cashflow!B9:M9)</f>
-        <v>233944</v>
+        <f aca="false">SUM(Cashflow!B7:M7)+Cashflow!O11</f>
+        <v>244093</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>233944</v>
+        <v>244093</v>
       </c>
       <c r="D23" s="5" t="n">
         <f aca="false">ROUND(B23-C23,2)</f>
@@ -1850,14 +1972,14 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B24" s="5" t="n">
-        <f aca="false">Cashflow!O13</f>
-        <v>81343.2</v>
+        <f aca="false">SUM(Cashflow!B8:M8)+Cashflow!O12</f>
+        <v>165246.3</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>81343.2</v>
+        <v>165246.3</v>
       </c>
       <c r="D24" s="5" t="n">
         <f aca="false">ROUND(B24-C24,2)</f>
@@ -1870,14 +1992,14 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B25" s="5" t="n">
-        <f aca="false">Cashflow!O14</f>
-        <v>724626.5</v>
+        <f aca="false">SUM(Cashflow!B9:M9)</f>
+        <v>233944</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>724626.5</v>
+        <v>233944</v>
       </c>
       <c r="D25" s="5" t="n">
         <f aca="false">ROUND(B25-C25,2)</f>
@@ -1890,14 +2012,14 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="B26" s="5" t="n">
-        <f aca="false">Cashflow!O16</f>
-        <v>705741.21</v>
+        <f aca="false">Cashflow!O13</f>
+        <v>81343.2</v>
       </c>
       <c r="C26" s="9" t="n">
-        <v>705741.21</v>
+        <v>81343.2</v>
       </c>
       <c r="D26" s="5" t="n">
         <f aca="false">ROUND(B26-C26,2)</f>
@@ -1910,14 +2032,14 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B27" s="5" t="n">
-        <f aca="false">Cashflow!O20</f>
-        <v>599880.03</v>
+        <f aca="false">Cashflow!O14</f>
+        <v>724626.5</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>599880.03</v>
+        <v>724626.5</v>
       </c>
       <c r="D27" s="5" t="n">
         <f aca="false">ROUND(B27-C27,2)</f>
@@ -1930,21 +2052,61 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="B28" s="5" t="n">
+        <f aca="false">Cashflow!O16</f>
+        <v>705741.21</v>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>705741.21</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <f aca="false">ROUND(B28-C28,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="8" t="str">
+        <f aca="false">IF(ABS(D28)&lt;=0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <f aca="false">Cashflow!O20</f>
+        <v>599880.03</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>599880.03</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <f aca="false">ROUND(B29-C29,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="8" t="str">
+        <f aca="false">IF(ABS(D29)&lt;=0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" s="5" t="n">
         <f aca="false">Cashflow!O14-Cashflow!O20</f>
         <v>124746.47</v>
       </c>
-      <c r="C28" s="9" t="n">
+      <c r="C30" s="9" t="n">
         <v>124746.47</v>
       </c>
-      <c r="D28" s="5" t="n">
-        <f aca="false">ROUND(B28-C28,2)</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="8" t="str">
-        <f aca="false">IF(ABS(D28)&lt;=0.05,"OK","SPRAWDŹ")</f>
+      <c r="D30" s="5" t="n">
+        <f aca="false">ROUND(B30-C30,2)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="8" t="str">
+        <f aca="false">IF(ABS(D30)&lt;=0.05,"OK","SPRAWDŹ")</f>
         <v>OK</v>
       </c>
     </row>
@@ -1977,99 +2139,121 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B4" s="10" t="n">
         <v>0.85</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>124746.47</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B9" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>55</v>
+      <c r="A11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -2091,57 +2275,57 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="J14" s="15" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="N14" s="15" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="P14" s="15" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>72966.67</v>
@@ -2192,7 +2376,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>9143.34</v>
@@ -2243,7 +2427,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D17" s="11" t="n">
         <v>0</v>
@@ -2288,12 +2472,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -2316,61 +2500,61 @@
     </row>
     <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="J21" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N21" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="O21" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="D21" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="E21" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="F21" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="G21" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="I21" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="J21" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="K21" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="L21" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="M21" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="N21" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="O21" s="16" t="s">
-        <v>70</v>
-      </c>
       <c r="P21" s="16" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="Q21" s="16" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="R21" s="16" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="S21" s="16" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2378,7 +2562,7 @@
         <v>1</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>14000</v>
@@ -2440,7 +2624,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>14000</v>
@@ -2502,7 +2686,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>14000</v>
@@ -2564,7 +2748,7 @@
         <v>1</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C25" s="9" t="n">
         <v>12048</v>
@@ -2626,7 +2810,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C26" s="9" t="n">
         <v>10000</v>
@@ -2688,7 +2872,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>14000</v>
@@ -2750,7 +2934,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>14000</v>
@@ -2812,7 +2996,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C29" s="9" t="n">
         <v>14000</v>
@@ -2874,7 +3058,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>14000</v>
@@ -2936,7 +3120,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>14000</v>
@@ -2998,7 +3182,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>14000</v>
@@ -3060,7 +3244,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>14000</v>
@@ -3122,7 +3306,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C34" s="9" t="n">
         <v>14000</v>
@@ -3184,7 +3368,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>12048</v>
@@ -3246,7 +3430,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C36" s="9" t="n">
         <v>10000</v>
@@ -3308,7 +3492,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C37" s="9" t="n">
         <v>14000</v>
@@ -3370,7 +3554,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C38" s="9" t="n">
         <v>14000</v>
@@ -3432,7 +3616,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C39" s="9" t="n">
         <v>14000</v>
@@ -3491,7 +3675,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="Q40" s="20" t="n">
         <f aca="false">SUM(Q22:Q39)</f>
@@ -3508,13 +3692,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B9" type="list">
-      <formula1>"1,2"</formula1>
+      <formula1>"1,2,3"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3533,7 +3717,346 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="70"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <f aca="false">Cashflow!B44</f>
+        <v>599880.03</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <f aca="false">ROUND(Założenia!B11*B4,2)</f>
+        <v>239952.01</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <f aca="false">ROUND(Założenia!B12*B4,2)</f>
+        <v>89982</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C9" s="4" t="str">
+        <f aca="false">Cashflow!B4</f>
+        <v>wrz 2026</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <f aca="false">Cashflow!B37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <f aca="false">D9/$B$4</f>
+        <v>0.399999996666</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <f aca="false">SUM($D$9:D9)</f>
+        <v>239952.01</v>
+      </c>
+      <c r="G9" s="22" t="n">
+        <f aca="false">F9/$B$4</f>
+        <v>0.399999996666</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <f aca="false">Cashflow!B39</f>
+        <v>239952.01</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" s="4" t="str">
+        <f aca="false">Cashflow!E4</f>
+        <v>gru 2026</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <f aca="false">Cashflow!E37</f>
+        <v>79244.76</v>
+      </c>
+      <c r="E10" s="22" t="n">
+        <f aca="false">D10/$B$4</f>
+        <v>0.132101013597669</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <f aca="false">SUM($D$9:D10)</f>
+        <v>319196.77</v>
+      </c>
+      <c r="G10" s="22" t="n">
+        <f aca="false">F10/$B$4</f>
+        <v>0.532101010263669</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <f aca="false">Cashflow!E39</f>
+        <v>153000.9705</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="4" t="str">
+        <f aca="false">Cashflow!H4</f>
+        <v>mar 2027</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <f aca="false">Cashflow!H37</f>
+        <v>145229.13</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <f aca="false">D11/$B$4</f>
+        <v>0.242096957286609</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <f aca="false">SUM($D$9:D11)</f>
+        <v>464425.9</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <f aca="false">F11/$B$4</f>
+        <v>0.774197967550278</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <f aca="false">Cashflow!H39</f>
+        <v>145229.1315</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="4" t="str">
+        <f aca="false">Cashflow!K4</f>
+        <v>cze 2027</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <f aca="false">Cashflow!K37</f>
+        <v>45472.13</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <f aca="false">D12/$B$4</f>
+        <v>0.0758020399512216</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <f aca="false">SUM($D$9:D12)</f>
+        <v>509898.03</v>
+      </c>
+      <c r="G12" s="22" t="n">
+        <f aca="false">F12/$B$4</f>
+        <v>0.8500000075015</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <f aca="false">Cashflow!K39</f>
+        <v>45472.1315</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C13" s="4" t="str">
+        <f aca="false">CHOOSE(Założenia!B10,"wrz 2027","paź 2027","lis 2027","gru 2027","sty 2028")</f>
+        <v>paź 2027</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <f aca="false">Cashflow!N37</f>
+        <v>89982</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <f aca="false">D13/$B$4</f>
+        <v>0.1499999924985</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <f aca="false">SUM($D$9:D13)</f>
+        <v>599880.03</v>
+      </c>
+      <c r="G13" s="22" t="n">
+        <f aca="false">F13/$B$4</f>
+        <v>1</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14" s="20" t="n">
+        <f aca="false">SUM(D9:D13)</f>
+        <v>599880.03</v>
+      </c>
+      <c r="E14" s="23" t="n">
+        <f aca="false">D14/B4</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <f aca="false">ROUND(D14-B4,2)</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="8" t="str">
+        <f aca="false">IF(ABS(B17)&lt;=0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <f aca="false">MAX(H9:H12)</f>
+        <v>239952.01</v>
+      </c>
+      <c r="C18" s="8" t="str">
+        <f aca="false">IF(B18&lt;=B5+0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <f aca="false">D13</f>
+        <v>89982</v>
+      </c>
+      <c r="C19" s="8" t="str">
+        <f aca="false">IF(D13&gt;=B6-0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <f aca="false">SUM(D9:D12)</f>
+        <v>509898.03</v>
+      </c>
+      <c r="C20" s="8" t="str">
+        <f aca="false">IF(B20&lt;=B4-B6+0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -3542,109 +4065,109 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="str">
-        <f aca="false">"Scenariusz wpływu dofinansowania: "&amp;IF(Założenia!B9=1,"1 – zaliczki kwartalne","2 – refundacja kwartalna z opóźnieniem "&amp;Założenia!B10&amp;" mies.")</f>
-        <v>Scenariusz wpływu dofinansowania: 1 – zaliczki kwartalne</v>
+      <c r="A2" s="24" t="str">
+        <f aca="false">"Scenariusz wpływu dofinansowania: "&amp;IF(Założenia!B9=1,"1 – zaliczki kwartalne",IF(Założenia!B9=2,"2 – refundacja kwartalna z opóźnieniem "&amp;Założenia!B10&amp;" mies.","3 – wg umowy: zaliczki (max "&amp;TEXT(Założenia!B11,"0%")&amp;") + płatność końcowa "&amp;TEXT(Założenia!B12,"0%")&amp;" po wniosku końcowym"))</f>
+        <v>Scenariusz wpływu dofinansowania: 3 – wg umowy: zaliczki (max 40%) + płatność końcowa 15% po wniosku końcowym</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="N4" s="16" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
       <c r="O4" s="16" t="s">
-        <v>95</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" s="22" t="n">
+        <v>131</v>
+      </c>
+      <c r="B5" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="D5" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="22" t="n">
+      <c r="E5" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="22" t="n">
+      <c r="F5" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="22" t="n">
+      <c r="L5" s="25" t="n">
         <v>11</v>
       </c>
-      <c r="M5" s="22" t="n">
+      <c r="M5" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="N5" s="22" t="n">
+      <c r="N5" s="25" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
@@ -3663,7 +4186,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">SUMPRODUCT((Założenia!$A$22:$A$39=1)*Założenia!D$22:D$39*Założenia!$C$22:$C$39)</f>
@@ -3723,7 +4246,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>99</v>
+        <v>134</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMPRODUCT((Założenia!$A$22:$A$39=2)*Założenia!D$22:D$39*Założenia!$C$22:$C$39)</f>
@@ -3783,7 +4306,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>100</v>
+        <v>135</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">SUMPRODUCT((Założenia!$A$22:$A$39=3)*Założenia!D$22:D$39*Założenia!$C$22:$C$39)</f>
@@ -3843,7 +4366,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>101</v>
+        <v>136</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">SUM(B7:B9)</f>
@@ -3893,7 +4416,7 @@
         <f aca="false">SUM(M7:M9)</f>
         <v>44524</v>
       </c>
-      <c r="N10" s="23" t="n">
+      <c r="N10" s="26" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="20" t="n">
@@ -3903,7 +4426,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>102</v>
+        <v>137</v>
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Założenia!$C$15*Założenia!D$15</f>
@@ -3963,7 +4486,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>103</v>
+        <v>138</v>
       </c>
       <c r="B12" s="5" t="n">
         <f aca="false">Założenia!$C$16*Założenia!D$16</f>
@@ -4023,7 +4546,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>104</v>
+        <v>139</v>
       </c>
       <c r="B13" s="5" t="n">
         <f aca="false">Założenia!$B$5*B10</f>
@@ -4083,7 +4606,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="B14" s="20" t="n">
         <f aca="false">SUM(B10:B13)</f>
@@ -4133,7 +4656,7 @@
         <f aca="false">SUM(M10:M13)</f>
         <v>51202.6</v>
       </c>
-      <c r="N14" s="23" t="n">
+      <c r="N14" s="26" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="20" t="n">
@@ -4143,7 +4666,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="B16" s="5" t="n">
         <f aca="false">B10+B13+Założenia!$B$15*Założenia!D$15+Założenia!$B$16*Założenia!D$16</f>
@@ -4203,7 +4726,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
       <c r="B17" s="5" t="n">
         <f aca="false">B14-B16</f>
@@ -4263,7 +4786,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>108</v>
+        <v>143</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -4282,59 +4805,59 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>109</v>
+        <v>144</v>
       </c>
       <c r="B20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,B33,B34)</f>
-        <v>166195.8</v>
+        <f aca="false">CHOOSE(Założenia!$B$9,B33,B34,B37)</f>
+        <v>239952.01</v>
       </c>
       <c r="C20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,C33,C34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,C33,C34,C37)</f>
         <v>0</v>
       </c>
       <c r="D20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,D33,D34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,D33,D34,D37)</f>
         <v>0</v>
       </c>
       <c r="E20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,E33,E34)</f>
-        <v>153000.97</v>
+        <f aca="false">CHOOSE(Założenia!$B$9,E33,E34,E37)</f>
+        <v>79244.76</v>
       </c>
       <c r="F20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,F33,F34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,F33,F34,F37)</f>
         <v>0</v>
       </c>
       <c r="G20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,G33,G34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,G33,G34,G37)</f>
         <v>0</v>
       </c>
       <c r="H20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,H33,H34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,H33,H34,H37)</f>
         <v>145229.13</v>
       </c>
       <c r="I20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,I33,I34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,I33,I34,I37)</f>
         <v>0</v>
       </c>
       <c r="J20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,J33,J34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,J33,J34,J37)</f>
         <v>0</v>
       </c>
       <c r="K20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,K33,K34)</f>
-        <v>135454.13</v>
+        <f aca="false">CHOOSE(Założenia!$B$9,K33,K34,K37)</f>
+        <v>45472.13</v>
       </c>
       <c r="L20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,L33,L34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,L33,L34,L37)</f>
         <v>0</v>
       </c>
       <c r="M20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,M33,M34)</f>
+        <f aca="false">CHOOSE(Założenia!$B$9,M33,M34,M37)</f>
         <v>0</v>
       </c>
       <c r="N20" s="5" t="n">
-        <f aca="false">CHOOSE(Założenia!$B$9,N33,N34)</f>
-        <v>0</v>
+        <f aca="false">CHOOSE(Założenia!$B$9,N33,N34,N37)</f>
+        <v>89982</v>
       </c>
       <c r="O20" s="20" t="n">
         <f aca="false">SUM(B20:N20)</f>
@@ -4343,53 +4866,53 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B21" s="24" t="n">
+        <v>145</v>
+      </c>
+      <c r="B21" s="27" t="n">
         <f aca="false">Założenia!D17</f>
         <v>0</v>
       </c>
-      <c r="C21" s="24" t="n">
+      <c r="C21" s="27" t="n">
         <f aca="false">Założenia!E17</f>
         <v>0</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="27" t="n">
         <f aca="false">Założenia!F17</f>
         <v>0</v>
       </c>
-      <c r="E21" s="24" t="n">
+      <c r="E21" s="27" t="n">
         <f aca="false">Założenia!G17</f>
         <v>0</v>
       </c>
-      <c r="F21" s="24" t="n">
+      <c r="F21" s="27" t="n">
         <f aca="false">Założenia!H17</f>
         <v>0</v>
       </c>
-      <c r="G21" s="24" t="n">
+      <c r="G21" s="27" t="n">
         <f aca="false">Założenia!I17</f>
         <v>0</v>
       </c>
-      <c r="H21" s="24" t="n">
+      <c r="H21" s="27" t="n">
         <f aca="false">Założenia!J17</f>
         <v>0</v>
       </c>
-      <c r="I21" s="24" t="n">
+      <c r="I21" s="27" t="n">
         <f aca="false">Założenia!K17</f>
         <v>0</v>
       </c>
-      <c r="J21" s="24" t="n">
+      <c r="J21" s="27" t="n">
         <f aca="false">Założenia!L17</f>
         <v>0</v>
       </c>
-      <c r="K21" s="24" t="n">
+      <c r="K21" s="27" t="n">
         <f aca="false">Założenia!M17</f>
         <v>0</v>
       </c>
-      <c r="L21" s="24" t="n">
+      <c r="L21" s="27" t="n">
         <f aca="false">Założenia!N17</f>
         <v>0</v>
       </c>
-      <c r="M21" s="24" t="n">
+      <c r="M21" s="27" t="n">
         <f aca="false">Założenia!O17</f>
         <v>0</v>
       </c>
@@ -4403,7 +4926,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>111</v>
+        <v>146</v>
       </c>
       <c r="B22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6,MAX(0,Założenia!$B$8-(B26+B20+B21-B14)))</f>
@@ -4415,7 +4938,7 @@
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:C22),MAX(0,Założenia!$B$8-(D26+D20+D21-D14)))</f>
-        <v>46111</v>
+        <v>0</v>
       </c>
       <c r="E22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:D22),MAX(0,Założenia!$B$8-(E26+E20+E21-E14)))</f>
@@ -4423,11 +4946,11 @@
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:E22),MAX(0,Założenia!$B$8-(F26+F20+F21-F14)))</f>
-        <v>0</v>
+        <v>18261.53</v>
       </c>
       <c r="G22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:F22),MAX(0,Założenia!$B$8-(G26+G20+G21-G14)))</f>
-        <v>29103.13</v>
+        <v>56952.6</v>
       </c>
       <c r="H22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:G22),MAX(0,Założenia!$B$8-(H26+H20+H21-H14)))</f>
@@ -4443,15 +4966,15 @@
       </c>
       <c r="K22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:J22),MAX(0,Założenia!$B$8-(K26+K20+K21-K14)))</f>
-        <v>0</v>
+        <v>11480.47</v>
       </c>
       <c r="L22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:K22),MAX(0,Założenia!$B$8-(L26+L20+L21-L14)))</f>
-        <v>0</v>
+        <v>12423.2</v>
       </c>
       <c r="M22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:L22),MAX(0,Założenia!$B$8-(M26+M20+M21-M14)))</f>
-        <v>23903.67</v>
+        <v>0</v>
       </c>
       <c r="N22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:M22),MAX(0,Założenia!$B$8-(N26+N20+N21-N14)))</f>
@@ -4464,11 +4987,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>166195.8</v>
+        <v>239952.01</v>
       </c>
       <c r="C23" s="20" t="n">
         <f aca="false">SUM(C20:C22)</f>
@@ -4476,19 +4999,19 @@
       </c>
       <c r="D23" s="20" t="n">
         <f aca="false">SUM(D20:D22)</f>
-        <v>46111</v>
+        <v>0</v>
       </c>
       <c r="E23" s="20" t="n">
         <f aca="false">SUM(E20:E22)</f>
-        <v>153000.97</v>
+        <v>79244.76</v>
       </c>
       <c r="F23" s="20" t="n">
         <f aca="false">SUM(F20:F22)</f>
-        <v>0</v>
+        <v>18261.53</v>
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">SUM(G20:G22)</f>
-        <v>29103.13</v>
+        <v>56952.6</v>
       </c>
       <c r="H23" s="20" t="n">
         <f aca="false">SUM(H20:H22)</f>
@@ -4504,19 +5027,19 @@
       </c>
       <c r="K23" s="20" t="n">
         <f aca="false">SUM(K20:K22)</f>
-        <v>135454.13</v>
+        <v>56952.6</v>
       </c>
       <c r="L23" s="20" t="n">
         <f aca="false">SUM(L20:L22)</f>
-        <v>0</v>
+        <v>12423.2</v>
       </c>
       <c r="M23" s="20" t="n">
         <f aca="false">SUM(M20:M22)</f>
-        <v>23903.67</v>
+        <v>0</v>
       </c>
       <c r="N23" s="20" t="n">
         <f aca="false">SUM(N20:N22)</f>
-        <v>0</v>
+        <v>89982</v>
       </c>
       <c r="O23" s="20" t="n">
         <f aca="false">SUM(B23:N23)</f>
@@ -4525,7 +5048,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>113</v>
+        <v>148</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -4544,7 +5067,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>114</v>
+        <v>149</v>
       </c>
       <c r="B26" s="5" t="n">
         <f aca="false">Założenia!$B$7</f>
@@ -4552,23 +5075,23 @@
       </c>
       <c r="C26" s="5" t="n">
         <f aca="false">B28</f>
-        <v>133393.2</v>
+        <v>207149.41</v>
       </c>
       <c r="D26" s="5" t="n">
         <f aca="false">C28</f>
-        <v>55716.1</v>
+        <v>129472.31</v>
       </c>
       <c r="E26" s="5" t="n">
         <f aca="false">D28</f>
-        <v>0</v>
+        <v>27645.21</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">E28</f>
-        <v>84802.07</v>
+        <v>38691.07</v>
       </c>
       <c r="G26" s="5" t="n">
         <f aca="false">F28</f>
-        <v>27849.47</v>
+        <v>0</v>
       </c>
       <c r="H26" s="5" t="n">
         <f aca="false">G28</f>
@@ -4588,15 +5111,15 @@
       </c>
       <c r="L26" s="5" t="n">
         <f aca="false">K28</f>
-        <v>78501.53</v>
+        <v>0</v>
       </c>
       <c r="M26" s="5" t="n">
         <f aca="false">L28</f>
-        <v>27298.93</v>
+        <v>-38779.4</v>
       </c>
       <c r="N26" s="5" t="n">
         <f aca="false">M28</f>
-        <v>0</v>
+        <v>-89982</v>
       </c>
       <c r="O26" s="20" t="n">
         <f aca="false">B26</f>
@@ -4605,11 +5128,11 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="B27" s="5" t="n">
         <f aca="false">B23-B14</f>
-        <v>133393.2</v>
+        <v>207149.41</v>
       </c>
       <c r="C27" s="5" t="n">
         <f aca="false">C23-C14</f>
@@ -4617,19 +5140,19 @@
       </c>
       <c r="D27" s="5" t="n">
         <f aca="false">D23-D14</f>
-        <v>-55716.1</v>
+        <v>-101827.1</v>
       </c>
       <c r="E27" s="5" t="n">
         <f aca="false">E23-E14</f>
-        <v>84802.07</v>
+        <v>11045.86</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">F23-F14</f>
-        <v>-56952.6</v>
+        <v>-38691.07</v>
       </c>
       <c r="G27" s="5" t="n">
         <f aca="false">G23-G14</f>
-        <v>-27849.47</v>
+        <v>0</v>
       </c>
       <c r="H27" s="5" t="n">
         <f aca="false">H23-H14</f>
@@ -4645,19 +5168,19 @@
       </c>
       <c r="K27" s="5" t="n">
         <f aca="false">K23-K14</f>
-        <v>78501.53</v>
+        <v>0</v>
       </c>
       <c r="L27" s="5" t="n">
         <f aca="false">L23-L14</f>
-        <v>-51202.6</v>
+        <v>-38779.4</v>
       </c>
       <c r="M27" s="5" t="n">
         <f aca="false">M23-M14</f>
-        <v>-27298.93</v>
+        <v>-51202.6</v>
       </c>
       <c r="N27" s="5" t="n">
         <f aca="false">N23-N14</f>
-        <v>0</v>
+        <v>89982</v>
       </c>
       <c r="O27" s="20" t="n">
         <f aca="false">SUM(B27:N27)</f>
@@ -4666,27 +5189,27 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>116</v>
+        <v>151</v>
       </c>
       <c r="B28" s="20" t="n">
         <f aca="false">B26+B27</f>
-        <v>133393.2</v>
+        <v>207149.41</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">C26+C27</f>
-        <v>55716.1</v>
+        <v>129472.31</v>
       </c>
       <c r="D28" s="20" t="n">
         <f aca="false">D26+D27</f>
-        <v>0</v>
+        <v>27645.21</v>
       </c>
       <c r="E28" s="20" t="n">
         <f aca="false">E26+E27</f>
-        <v>84802.07</v>
+        <v>38691.07</v>
       </c>
       <c r="F28" s="20" t="n">
         <f aca="false">F26+F27</f>
-        <v>27849.47</v>
+        <v>0</v>
       </c>
       <c r="G28" s="20" t="n">
         <f aca="false">G26+G27</f>
@@ -4706,15 +5229,15 @@
       </c>
       <c r="K28" s="20" t="n">
         <f aca="false">K26+K27</f>
-        <v>78501.53</v>
+        <v>0</v>
       </c>
       <c r="L28" s="20" t="n">
         <f aca="false">L26+L27</f>
-        <v>27298.93</v>
+        <v>-38779.4</v>
       </c>
       <c r="M28" s="20" t="n">
         <f aca="false">M26+M27</f>
-        <v>0</v>
+        <v>-89982</v>
       </c>
       <c r="N28" s="20" t="n">
         <f aca="false">N26+N27</f>
@@ -4727,7 +5250,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>117</v>
+        <v>152</v>
       </c>
       <c r="B29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-B28)</f>
@@ -4771,11 +5294,11 @@
       </c>
       <c r="L29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-L28)</f>
-        <v>0</v>
+        <v>38779.4</v>
       </c>
       <c r="M29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-M28)</f>
-        <v>0</v>
+        <v>89982</v>
       </c>
       <c r="N29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-N28)</f>
@@ -4783,12 +5306,12 @@
       </c>
       <c r="O29" s="20" t="n">
         <f aca="false">MAX(B29:N29)</f>
-        <v>0</v>
+        <v>89982</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>153</v>
       </c>
       <c r="B30" s="5" t="n">
         <f aca="false">SUM($B22:B22)</f>
@@ -4800,15 +5323,15 @@
       </c>
       <c r="D30" s="5" t="n">
         <f aca="false">SUM($B22:D22)</f>
-        <v>46111</v>
+        <v>0</v>
       </c>
       <c r="E30" s="5" t="n">
         <f aca="false">SUM($B22:E22)</f>
-        <v>46111</v>
+        <v>0</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">SUM($B22:F22)</f>
-        <v>46111</v>
+        <v>18261.53</v>
       </c>
       <c r="G30" s="5" t="n">
         <f aca="false">SUM($B22:G22)</f>
@@ -4828,11 +5351,11 @@
       </c>
       <c r="K30" s="5" t="n">
         <f aca="false">SUM($B22:K22)</f>
-        <v>100842.8</v>
+        <v>112323.27</v>
       </c>
       <c r="L30" s="5" t="n">
         <f aca="false">SUM($B22:L22)</f>
-        <v>100842.8</v>
+        <v>124746.47</v>
       </c>
       <c r="M30" s="5" t="n">
         <f aca="false">SUM($B22:M22)</f>
@@ -4849,7 +5372,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>119</v>
+        <v>154</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -4868,7 +5391,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="B33" s="5" t="n">
         <f aca="false">IF(MOD(B$5-1,3)=0,ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;B$5,$B$5:$M$5,"&lt;="&amp;(B$5+2)),2),0)</f>
@@ -4929,7 +5452,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>121</v>
+        <v>156</v>
       </c>
       <c r="B34" s="5" t="n">
         <f aca="false">IF(AND(B$5-Założenia!$B$10&gt;=3,MOD(B$5-Założenia!$B$10,3)=0),ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;"&amp;(B$5-Założenia!$B$10-3),$B$5:$M$5,"&lt;="&amp;(B$5-Założenia!$B$10)),2),0)</f>
@@ -4990,7 +5513,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>122</v>
+        <v>157</v>
       </c>
       <c r="B35" s="5" t="n">
         <f aca="false">Założenia!$B$7+B33+B21-B14</f>
@@ -5047,7 +5570,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="B36" s="5" t="n">
         <f aca="false">Założenia!$B$7+B34+B21-B14</f>
@@ -5102,9 +5625,362 @@
         <v>-124746.47</v>
       </c>
     </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <f aca="false">MIN(ROUND(Założenia!$B$11*$B$44,2),ROUND((1-Założenia!$B$12)*$B$44,2))</f>
+        <v>239952.01</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <f aca="false">IF(MOD(C$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-B41,Założenia!$B$11*$B$44-C42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;C$5,$B$5:$M$5,"&lt;="&amp;(C$5+2))-C42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <f aca="false">IF(MOD(D$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-C41,Założenia!$B$11*$B$44-D42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;D$5,$B$5:$M$5,"&lt;="&amp;(D$5+2))-D42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <f aca="false">IF(MOD(E$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-D41,Założenia!$B$11*$B$44-E42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;E$5,$B$5:$M$5,"&lt;="&amp;(E$5+2))-E42)),2),0)</f>
+        <v>79244.76</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <f aca="false">IF(MOD(F$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-E41,Założenia!$B$11*$B$44-F42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;F$5,$B$5:$M$5,"&lt;="&amp;(F$5+2))-F42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <f aca="false">IF(MOD(G$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-F41,Założenia!$B$11*$B$44-G42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;G$5,$B$5:$M$5,"&lt;="&amp;(G$5+2))-G42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <f aca="false">IF(MOD(H$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-G41,Założenia!$B$11*$B$44-H42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;H$5,$B$5:$M$5,"&lt;="&amp;(H$5+2))-H42)),2),0)</f>
+        <v>145229.13</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <f aca="false">IF(MOD(I$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-H41,Założenia!$B$11*$B$44-I42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;I$5,$B$5:$M$5,"&lt;="&amp;(I$5+2))-I42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <f aca="false">IF(MOD(J$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-I41,Założenia!$B$11*$B$44-J42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;J$5,$B$5:$M$5,"&lt;="&amp;(J$5+2))-J42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <f aca="false">IF(MOD(K$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-J41,Założenia!$B$11*$B$44-K42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;K$5,$B$5:$M$5,"&lt;="&amp;(K$5+2))-K42)),2),0)</f>
+        <v>45472.13</v>
+      </c>
+      <c r="L37" s="5" t="n">
+        <f aca="false">IF(MOD(L$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-K41,Założenia!$B$11*$B$44-L42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;L$5,$B$5:$M$5,"&lt;="&amp;(L$5+2))-L42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M37" s="5" t="n">
+        <f aca="false">IF(MOD(M$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-L41,Założenia!$B$11*$B$44-M42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;M$5,$B$5:$M$5,"&lt;="&amp;(M$5+2))-M42)),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="N37" s="5" t="n">
+        <f aca="false">$B$44-SUM(B37:M37)</f>
+        <v>89982</v>
+      </c>
+      <c r="O37" s="20" t="n">
+        <f aca="false">SUM(B37:N37)</f>
+        <v>599880.03</v>
+      </c>
+    </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
-        <v>124</v>
+      <c r="A38" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B38" s="5" t="n">
+        <f aca="false">Założenia!$B$7+B37+B21-B14</f>
+        <v>207149.41</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <f aca="false">B38+C37+C21-C14</f>
+        <v>129472.31</v>
+      </c>
+      <c r="D38" s="5" t="n">
+        <f aca="false">C38+D37+D21-D14</f>
+        <v>27645.21</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <f aca="false">D38+E37+E21-E14</f>
+        <v>38691.07</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <f aca="false">E38+F37+F21-F14</f>
+        <v>-18261.53</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <f aca="false">F38+G37+G21-G14</f>
+        <v>-75214.13</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <f aca="false">G38+H37+H21-H14</f>
+        <v>13062.4</v>
+      </c>
+      <c r="I38" s="5" t="n">
+        <f aca="false">H38+I37+I21-I14</f>
+        <v>-43890.2</v>
+      </c>
+      <c r="J38" s="5" t="n">
+        <f aca="false">I38+J37+J21-J14</f>
+        <v>-100842.8</v>
+      </c>
+      <c r="K38" s="5" t="n">
+        <f aca="false">J38+K37+K21-K14</f>
+        <v>-112323.27</v>
+      </c>
+      <c r="L38" s="5" t="n">
+        <f aca="false">K38+L37+L21-L14</f>
+        <v>-163525.87</v>
+      </c>
+      <c r="M38" s="5" t="n">
+        <f aca="false">L38+M37+M21-M14</f>
+        <v>-214728.47</v>
+      </c>
+      <c r="N38" s="5" t="n">
+        <f aca="false">M38+N37+N21-N14</f>
+        <v>-124746.47</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B39" s="5" t="n">
+        <f aca="false">B42+B37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <f aca="false">C42+C37</f>
+        <v>212069.8</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <f aca="false">D42+D37</f>
+        <v>153176.75525</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <f aca="false">E42+E37</f>
+        <v>153000.9705</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <f aca="false">F42+F37</f>
+        <v>96819.4215</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <f aca="false">G42+G37</f>
+        <v>48409.7115</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <f aca="false">H42+H37</f>
+        <v>145229.1315</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <f aca="false">I42+I37</f>
+        <v>96819.4215000001</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <f aca="false">J42+J37</f>
+        <v>48409.7115000001</v>
+      </c>
+      <c r="K39" s="5" t="n">
+        <f aca="false">K42+K37</f>
+        <v>45472.1315</v>
+      </c>
+      <c r="L39" s="5" t="n">
+        <f aca="false">L42+L37</f>
+        <v>0</v>
+      </c>
+      <c r="M39" s="5" t="n">
+        <f aca="false">M42+M37</f>
+        <v>0</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B40" s="5" t="n">
+        <f aca="false">SUM($B16:B16)</f>
+        <v>32802.6</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <f aca="false">SUM($B16:C16)</f>
+        <v>102088.535</v>
+      </c>
+      <c r="D40" s="5" t="n">
+        <f aca="false">SUM($B16:D16)</f>
+        <v>195524.47</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <f aca="false">SUM($B16:E16)</f>
+        <v>261620.41</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <f aca="false">SUM($B16:F16)</f>
+        <v>318573.01</v>
+      </c>
+      <c r="G40" s="5" t="n">
+        <f aca="false">SUM($B16:G16)</f>
+        <v>375525.61</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <f aca="false">SUM($B16:H16)</f>
+        <v>432478.21</v>
+      </c>
+      <c r="I40" s="5" t="n">
+        <f aca="false">SUM($B16:I16)</f>
+        <v>489430.81</v>
+      </c>
+      <c r="J40" s="5" t="n">
+        <f aca="false">SUM($B16:J16)</f>
+        <v>546383.41</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <f aca="false">SUM($B16:K16)</f>
+        <v>603336.01</v>
+      </c>
+      <c r="L40" s="5" t="n">
+        <f aca="false">SUM($B16:L16)</f>
+        <v>654538.61</v>
+      </c>
+      <c r="M40" s="5" t="n">
+        <f aca="false">SUM($B16:M16)</f>
+        <v>705741.21</v>
+      </c>
+      <c r="N40" s="5" t="n">
+        <f aca="false">SUM($B16:N16)</f>
+        <v>705741.21</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B41" s="5" t="n">
+        <f aca="false">B37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <f aca="false">B41+C37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <f aca="false">C41+D37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <f aca="false">D41+E37</f>
+        <v>319196.77</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <f aca="false">E41+F37</f>
+        <v>319196.77</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <f aca="false">F41+G37</f>
+        <v>319196.77</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <f aca="false">G41+H37</f>
+        <v>464425.9</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <f aca="false">H41+I37</f>
+        <v>464425.9</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <f aca="false">I41+J37</f>
+        <v>464425.9</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <f aca="false">J41+K37</f>
+        <v>509898.03</v>
+      </c>
+      <c r="L41" s="5" t="n">
+        <f aca="false">K41+L37</f>
+        <v>509898.03</v>
+      </c>
+      <c r="M41" s="5" t="n">
+        <f aca="false">L41+M37</f>
+        <v>509898.03</v>
+      </c>
+      <c r="N41" s="5" t="n">
+        <f aca="false">M41+N37</f>
+        <v>599880.03</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <f aca="false">MAX(0,B41-Założenia!$B$4*B40)</f>
+        <v>212069.8</v>
+      </c>
+      <c r="D42" s="5" t="n">
+        <f aca="false">MAX(0,C41-Założenia!$B$4*C40)</f>
+        <v>153176.75525</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <f aca="false">MAX(0,D41-Założenia!$B$4*D40)</f>
+        <v>73756.2105</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <f aca="false">MAX(0,E41-Założenia!$B$4*E40)</f>
+        <v>96819.4215</v>
+      </c>
+      <c r="G42" s="5" t="n">
+        <f aca="false">MAX(0,F41-Założenia!$B$4*F40)</f>
+        <v>48409.7115</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <f aca="false">MAX(0,G41-Założenia!$B$4*G40)</f>
+        <v>0.00150000001303852</v>
+      </c>
+      <c r="I42" s="5" t="n">
+        <f aca="false">MAX(0,H41-Założenia!$B$4*H40)</f>
+        <v>96819.4215000001</v>
+      </c>
+      <c r="J42" s="5" t="n">
+        <f aca="false">MAX(0,I41-Założenia!$B$4*I40)</f>
+        <v>48409.7115000001</v>
+      </c>
+      <c r="K42" s="5" t="n">
+        <f aca="false">MAX(0,J41-Założenia!$B$4*J40)</f>
+        <v>0.00150000001303852</v>
+      </c>
+      <c r="L42" s="5" t="n">
+        <f aca="false">MAX(0,K41-Założenia!$B$4*K40)</f>
+        <v>0</v>
+      </c>
+      <c r="M42" s="5" t="n">
+        <f aca="false">MAX(0,L41-Założenia!$B$4*L40)</f>
+        <v>0</v>
+      </c>
+      <c r="N42" s="5" t="n">
+        <f aca="false">MAX(0,M41-Założenia!$B$4*M40)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <f aca="false">ROUND(Założenia!$B$4*SUM($B$16:$M$16),2)</f>
+        <v>599880.03</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Przelicz harmonogram płatności (zaliczka 40%, kolejna po wydatkowaniu 70%) i wypełnij wzór HP PARP
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Av3yRtjc51k31HhvjViJWB
</commit_message>
<xml_diff>
--- a/Cashflow_SZMO.xlsx
+++ b/Cashflow_SZMO.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Założenia" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Harmonogram płatności" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Cashflow" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="HP – wzór PARP" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="201">
   <si>
     <t xml:space="preserve">Cashflow projektu SZMO – podsumowanie</t>
   </si>
@@ -160,30 +161,45 @@
     <t xml:space="preserve">Scen. 1: zaliczka na początku kwartału = 85% kosztów kwalif. kolejnych 3 mies. | Scen. 2: refundacja 85% kosztów kwartału z opóźnieniem | Scen. 3: 1. zaliczka = max % z B11, kolejne zaliczki kwartalnie wg potrzeb (niewykorzystana zaliczka ≤ B11, łącznie ≤ 100% − B12), reszta po wniosku końcowym.</t>
   </si>
   <si>
+    <t xml:space="preserve">Parametry scenariusza 3 (zaliczki wg umowy)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stopa dofinansowania</t>
   </si>
   <si>
     <t xml:space="preserve">Wniosek – podsumowanie wydatków</t>
   </si>
   <si>
+    <t xml:space="preserve">Miesiąc wypłaty 1. zaliczki (nr mies.: 1 = wrz 2026, 3 = lis 2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Stawka kosztów pośrednich (od wynagrodzeń kwalifik.)</t>
   </si>
   <si>
     <t xml:space="preserve">Wniosek – koszty uproszczone (ryczałt 15%)</t>
   </si>
   <si>
+    <t xml:space="preserve">Kolejna zaliczka po wydatkowaniu min. % wypłaconych narastająco</t>
+  </si>
+  <si>
     <t xml:space="preserve">Limit pożyczek właścicielskich (wkład własny, PLN)</t>
   </si>
   <si>
     <t xml:space="preserve">Wniosek – źródła finansowania (pożyczka, przedwstępne umowy)</t>
   </si>
   <si>
+    <t xml:space="preserve">Opóźnienie rozliczenia wydatków przed kolejną zaliczką (mies.)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Saldo początkowe gotówki (PLN)</t>
   </si>
   <si>
     <t xml:space="preserve">ZAŁOŻENIE – brak danych we wniosku</t>
   </si>
   <si>
+    <t xml:space="preserve">Wydatkowanie liczone jako 85% × wydatki kwalifikowalne narastająco od początku projektu (w tym wrz–paź 2026).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Minimalne saldo gotówki / bufor (PLN)</t>
   </si>
   <si>
@@ -202,7 +218,7 @@
     <t xml:space="preserve">ZAŁOŻENIE – dot. scenariuszy 2 i 3 (od końca kwartału / od końca projektu)</t>
   </si>
   <si>
-    <t xml:space="preserve">Maksymalna zaliczka (% dofinansowania) – scen. 3</t>
+    <t xml:space="preserve">Maksymalna pojedyncza zaliczka (% dofinansowania) – scen. 3</t>
   </si>
   <si>
     <t xml:space="preserve">UMOWA O DOFINANSOWANIE: zaliczka maks. 40% dofinansowania</t>
@@ -328,7 +344,7 @@
     <t xml:space="preserve">Harmonogram płatności dofinansowania – wg zapisów umowy</t>
   </si>
   <si>
-    <t xml:space="preserve">Zaliczka maks. 40% dofinansowania; 15% dofinansowania wypłacane w formie refundacji po wniosku o płatność końcową. Terminy kwartalnych zaliczek i opóźnienie płatności końcowej to założenia (Założenia!B10). Arkusz zawsze pokazuje scenariusz 3, niezależnie od wyboru w Założeniach.</t>
+    <t xml:space="preserve">Zaliczka maks. 40% dofinansowania; kolejna zaliczka dopiero po wydatkowaniu 70% wypłaconych dotąd zaliczek (narastająco); 15% dofinansowania wypłacane w formie refundacji po wniosku o płatność końcową (opóźnienie – Założenia!B10). Arkusz zawsze pokazuje scenariusz 3, niezależnie od wyboru w Założeniach.</t>
   </si>
   <si>
     <t xml:space="preserve">Dofinansowanie ogółem (PLN)</t>
@@ -364,28 +380,34 @@
     <t xml:space="preserve">Niewykorzystana zaliczka po wypłacie (PLN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Zaliczka nr 1 – na start projektu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pierwsza zaliczka w maksymalnej wysokości 40% dofinansowania</t>
+    <t xml:space="preserve">Wydatkowano z wcześniej wypłaconych (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaliczka nr 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maksymalna zaliczka (40% dofinansowania), wypłata na początku miesiąca</t>
   </si>
   <si>
     <t xml:space="preserve">Zaliczka nr 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Uzupełnienie zaliczki na potrzeby kolejnego kwartału (po rozliczeniu wydatków)</t>
+    <t xml:space="preserve">Po wydatkowaniu min. 70% wypłaconych dotąd zaliczek – kwota wg limitu 40%</t>
   </si>
   <si>
     <t xml:space="preserve">Zaliczka nr 3</t>
   </si>
   <si>
-    <t xml:space="preserve">jw.</t>
+    <t xml:space="preserve">Domknięcie limitu 85% (zaliczki + refundacje przed wnioskiem końcowym) po wydatkowaniu 70%</t>
   </si>
   <si>
     <t xml:space="preserve">Zaliczka nr 4</t>
   </si>
   <si>
-    <t xml:space="preserve">jw.; łącznie zaliczki i płatności pośrednie ≤ 85% dofinansowania</t>
+    <t xml:space="preserve">Nie występuje (limit 85% wykorzystany)</t>
   </si>
   <si>
     <t xml:space="preserve">Płatność końcowa (refundacja po wniosku o płatność końcową)</t>
@@ -400,7 +422,7 @@
     <t xml:space="preserve">Suma płatności = dofinansowanie</t>
   </si>
   <si>
-    <t xml:space="preserve">Najwyższa niewykorzystana zaliczka ≤ 40% dofinansowania</t>
+    <t xml:space="preserve">Największa pojedyncza zaliczka ≤ 40% dofinansowania</t>
   </si>
   <si>
     <t xml:space="preserve">Płatność końcowa ≥ 15% dofinansowania</t>
@@ -409,6 +431,9 @@
     <t xml:space="preserve">Wypłaty przed wnioskiem końcowym ≤ 85% dofinansowania</t>
   </si>
   <si>
+    <t xml:space="preserve">Kolejna zaliczka po wydatkowaniu ≥ 70% wypłaconych dotąd (najniższe wydatkowanie)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cashflow projektu SZMO – miesięcznie (PLN)</t>
   </si>
   <si>
@@ -520,10 +545,88 @@
     <t xml:space="preserve">Niewykorzystana zaliczka na początek miesiąca (scen. 3)</t>
   </si>
   <si>
+    <t xml:space="preserve">Nr zaliczki (scen. 3)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dofinansowanie ogółem (zaokrąglone)</t>
   </si>
   <si>
     <t xml:space="preserve">Pożyczka właścicielska jest uruchamiana automatycznie tylko do poziomu niedoboru gotówki (do limitu z Założeń); spłata pożyczek wspólnikom nie jest w modelu (brak informacji we wniosku). Kolumna „Po projekcie” to wpływy po 31.08.2027 (np. rozliczenie ostatniej transzy).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dane do Harmonogramu nr 1 (wzór PARP) – wartości z modelu, scenariusz 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numer Projektu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nazwa realizatora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rok</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kwartał</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miesiąc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dofinansowanie - zaliczka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dofinansowanie - refundacja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FEPW.01.01-IP.01-0825/26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMART-ELIT SP. Z O.O.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">listopad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">grudzień</t>
+  </si>
+  <si>
+    <t xml:space="preserve">styczeń</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marzec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kwiecień</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">czerwiec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lipiec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sierpień</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wrzesień</t>
+  </si>
+  <si>
+    <t xml:space="preserve">październik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrola: wydatki kwalifikowalne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kontrola: zaliczki + refundacja = dofinansowanie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wzór PARP zaczyna się od listopada 2026 – wydatki z wrz–paź 2026 ujęto w wierszu „listopad”. Płatność końcowa w „wrzesień/październik 2027” zależy od Założenia!B10 (1 lub 2). Wartości zostały przeniesione do osobnego pliku według wzoru.</t>
   </si>
 </sst>
 </file>
@@ -700,7 +803,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -745,11 +848,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -787,6 +890,10 @@
     </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -1167,34 +1274,34 @@
                 <c:formatCode>#,##0.00;[RED]\(#,##0.00\);\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
+                  <c:v>32802.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>77677.1</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>239952.01</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="4">
+                  <c:v>239952.01</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>79244.76</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>18261.53</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>56952.6</c:v>
-                </c:pt>
                 <c:pt idx="6">
-                  <c:v>145229.13</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
+                  <c:v>29994.01</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="8">
-                  <c:v>25628.67</c:v>
-                </c:pt>
                 <c:pt idx="9">
-                  <c:v>56952.6</c:v>
+                  <c:v>1843.57000000002</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>12423.2</c:v>
@@ -1208,8 +1315,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71421515"/>
-        <c:axId val="69056934"/>
+        <c:axId val="82546140"/>
+        <c:axId val="10554548"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1318,31 +1425,31 @@
                 <c:formatCode>#,##0.00;[RED]\(#,##0.00\);\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>207149.41</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>129472.31</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>27645.21</c:v>
+                  <c:v>138124.91</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>38691.07</c:v>
+                  <c:v>69926.01</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>252925.42</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>195972.82</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>88276.53</c:v>
+                  <c:v>139020.22</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>31323.93</c:v>
+                  <c:v>112061.63</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>55109.03</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -1366,11 +1473,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="71421515"/>
-        <c:axId val="69056934"/>
+        <c:axId val="82546140"/>
+        <c:axId val="10554548"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="71421515"/>
+        <c:axId val="82546140"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1402,7 +1509,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69056934"/>
+        <c:crossAx val="10554548"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1410,7 +1517,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69056934"/>
+        <c:axId val="10554548"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1452,7 +1559,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71421515"/>
+        <c:crossAx val="82546140"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2151,109 +2258,133 @@
       <c r="A3" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="E3" s="8" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" s="10" t="n">
         <v>0.85</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="L5" s="10" t="n">
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="11" t="n">
+        <v>52</v>
+      </c>
+      <c r="B6" s="12" t="n">
         <v>124746.47</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B7" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="B7" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="11" t="n">
+        <v>58</v>
+      </c>
+      <c r="B8" s="12" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B9" s="12" t="n">
+        <v>60</v>
+      </c>
+      <c r="B9" s="11" t="n">
         <v>3</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" s="12" t="n">
+        <v>62</v>
+      </c>
+      <c r="B10" s="11" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>0.4</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -2278,54 +2409,54 @@
         <v>29</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J14" s="15" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="K14" s="15" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="N14" s="15" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="P14" s="15" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B15" s="9" t="n">
         <v>72966.67</v>
@@ -2376,7 +2507,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B16" s="9" t="n">
         <v>9143.34</v>
@@ -2427,42 +2558,42 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="11" t="n">
+        <v>86</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="12" t="n">
         <v>0</v>
       </c>
       <c r="P17" s="5" t="n">
@@ -2472,12 +2603,12 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -2500,58 +2631,58 @@
     </row>
     <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="F21" s="16" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="J21" s="16" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="K21" s="16" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L21" s="16" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="N21" s="16" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="O21" s="16" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="P21" s="16" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="Q21" s="16" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="R21" s="16" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="S21" s="16" t="s">
         <v>32</v>
@@ -2562,7 +2693,7 @@
         <v>1</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>14000</v>
@@ -2624,7 +2755,7 @@
         <v>1</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C23" s="9" t="n">
         <v>14000</v>
@@ -2686,7 +2817,7 @@
         <v>1</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>14000</v>
@@ -2748,7 +2879,7 @@
         <v>1</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C25" s="9" t="n">
         <v>12048</v>
@@ -2810,7 +2941,7 @@
         <v>1</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C26" s="9" t="n">
         <v>10000</v>
@@ -2872,7 +3003,7 @@
         <v>2</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C27" s="9" t="n">
         <v>14000</v>
@@ -2934,7 +3065,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>14000</v>
@@ -2996,7 +3127,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C29" s="9" t="n">
         <v>14000</v>
@@ -3058,7 +3189,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>14000</v>
@@ -3120,7 +3251,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>14000</v>
@@ -3182,7 +3313,7 @@
         <v>3</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>14000</v>
@@ -3244,7 +3375,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>14000</v>
@@ -3306,7 +3437,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C34" s="9" t="n">
         <v>14000</v>
@@ -3368,7 +3499,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>12048</v>
@@ -3430,7 +3561,7 @@
         <v>3</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C36" s="9" t="n">
         <v>10000</v>
@@ -3492,7 +3623,7 @@
         <v>3</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C37" s="9" t="n">
         <v>14000</v>
@@ -3554,7 +3685,7 @@
         <v>3</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C38" s="9" t="n">
         <v>14000</v>
@@ -3616,7 +3747,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C39" s="9" t="n">
         <v>14000</v>
@@ -3675,7 +3806,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="Q40" s="20" t="n">
         <f aca="false">SUM(Q22:Q39)</f>
@@ -3692,7 +3823,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3717,7 +3848,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -3726,23 +3857,23 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="80"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B4" s="5" t="n">
         <f aca="false">Cashflow!B44</f>
@@ -3751,7 +3882,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">ROUND(Założenia!B11*B4,2)</f>
@@ -3760,7 +3891,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">ROUND(Założenia!B12*B4,2)</f>
@@ -3769,30 +3900,33 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="I8" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="J8" s="16" t="s">
         <v>4</v>
       </c>
     </row>
@@ -3801,17 +3935,17 @@
         <v>1</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="4" t="str">
-        <f aca="false">Cashflow!B4</f>
-        <v>wrz 2026</v>
+        <v>119</v>
+      </c>
+      <c r="C9" s="22" t="str">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$4:$M$4,MATCH(1,Cashflow!$B$43:$M$43,0)),"–")</f>
+        <v>lis 2026</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">Cashflow!B37</f>
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$37:$M$37,MATCH(1,Cashflow!$B$43:$M$43,0)),0)</f>
         <v>239952.01</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="23" t="n">
         <f aca="false">D9/$B$4</f>
         <v>0.399999996666</v>
       </c>
@@ -3819,16 +3953,19 @@
         <f aca="false">SUM($D$9:D9)</f>
         <v>239952.01</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="23" t="n">
         <f aca="false">F9/$B$4</f>
         <v>0.399999996666</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">Cashflow!B39</f>
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$39:$M$39,MATCH(1,Cashflow!$B$43:$M$43,0)),0)</f>
         <v>239952.01</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>114</v>
+      <c r="I9" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3836,34 +3973,38 @@
         <v>2</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C10" s="4" t="str">
-        <f aca="false">Cashflow!E4</f>
-        <v>gru 2026</v>
+        <v>122</v>
+      </c>
+      <c r="C10" s="22" t="str">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$4:$M$4,MATCH(2,Cashflow!$B$43:$M$43,0)),"–")</f>
+        <v>sty 2027</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">Cashflow!E37</f>
-        <v>79244.76</v>
-      </c>
-      <c r="E10" s="22" t="n">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$37:$M$37,MATCH(2,Cashflow!$B$43:$M$43,0)),0)</f>
+        <v>239952.01</v>
+      </c>
+      <c r="E10" s="23" t="n">
         <f aca="false">D10/$B$4</f>
-        <v>0.132101013597669</v>
+        <v>0.399999996666</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">SUM($D$9:D10)</f>
-        <v>319196.77</v>
-      </c>
-      <c r="G10" s="22" t="n">
+        <v>479904.02</v>
+      </c>
+      <c r="G10" s="23" t="n">
         <f aca="false">F10/$B$4</f>
-        <v>0.532101010263669</v>
+        <v>0.799999993332</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">Cashflow!E39</f>
-        <v>153000.9705</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>116</v>
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$39:$M$39,MATCH(2,Cashflow!$B$43:$M$43,0)),0)</f>
+        <v>257526.6715</v>
+      </c>
+      <c r="I10" s="23" t="n">
+        <f aca="false">IFERROR(Założenia!$B$4*INDEX(Cashflow!$B$40:$M$40,MATCH(2,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/F9,"–")</f>
+        <v>0.926757598321431</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3871,34 +4012,38 @@
         <v>3</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="C11" s="4" t="str">
-        <f aca="false">Cashflow!H4</f>
-        <v>mar 2027</v>
+        <v>124</v>
+      </c>
+      <c r="C11" s="22" t="str">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$4:$M$4,MATCH(3,Cashflow!$B$43:$M$43,0)),"–")</f>
+        <v>kwi 2027</v>
       </c>
       <c r="D11" s="5" t="n">
-        <f aca="false">Cashflow!H37</f>
-        <v>145229.13</v>
-      </c>
-      <c r="E11" s="22" t="n">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$37:$M$37,MATCH(3,Cashflow!$B$43:$M$43,0)),0)</f>
+        <v>29994.01</v>
+      </c>
+      <c r="E11" s="23" t="n">
         <f aca="false">D11/$B$4</f>
-        <v>0.242096957286609</v>
+        <v>0.0500000141694999</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">SUM($D$9:D11)</f>
-        <v>464425.9</v>
-      </c>
-      <c r="G11" s="22" t="n">
+        <v>509898.03</v>
+      </c>
+      <c r="G11" s="23" t="n">
         <f aca="false">F11/$B$4</f>
-        <v>0.774197967550278</v>
+        <v>0.8500000075015</v>
       </c>
       <c r="H11" s="5" t="n">
-        <f aca="false">Cashflow!H39</f>
-        <v>145229.1315</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>118</v>
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$39:$M$39,MATCH(3,Cashflow!$B$43:$M$43,0)),0)</f>
+        <v>142291.5515</v>
+      </c>
+      <c r="I11" s="23" t="n">
+        <f aca="false">IFERROR(Założenia!$B$4*INDEX(Cashflow!$B$40:$M$40,MATCH(3,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/F10,"–")</f>
+        <v>0.765999998291325</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3906,34 +4051,38 @@
         <v>4</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C12" s="4" t="str">
-        <f aca="false">Cashflow!K4</f>
-        <v>cze 2027</v>
+        <v>126</v>
+      </c>
+      <c r="C12" s="22" t="str">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$4:$M$4,MATCH(4,Cashflow!$B$43:$M$43,0)),"–")</f>
+        <v>–</v>
       </c>
       <c r="D12" s="5" t="n">
-        <f aca="false">Cashflow!K37</f>
-        <v>45472.13</v>
-      </c>
-      <c r="E12" s="22" t="n">
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$37:$M$37,MATCH(4,Cashflow!$B$43:$M$43,0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="23" t="n">
         <f aca="false">D12/$B$4</f>
-        <v>0.0758020399512216</v>
+        <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">SUM($D$9:D12)</f>
         <v>509898.03</v>
       </c>
-      <c r="G12" s="22" t="n">
+      <c r="G12" s="23" t="n">
         <f aca="false">F12/$B$4</f>
         <v>0.8500000075015</v>
       </c>
       <c r="H12" s="5" t="n">
-        <f aca="false">Cashflow!K39</f>
-        <v>45472.1315</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>120</v>
+        <f aca="false">IFERROR(INDEX(Cashflow!$B$39:$M$39,MATCH(4,Cashflow!$B$43:$M$43,0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="23" t="str">
+        <f aca="false">IFERROR(Założenia!$B$4*INDEX(Cashflow!$B$40:$M$40,MATCH(4,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/F11,"–")</f>
+        <v>–</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3941,7 +4090,7 @@
         <v>5</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C13" s="4" t="str">
         <f aca="false">CHOOSE(Założenia!B10,"wrz 2027","paź 2027","lis 2027","gru 2027","sty 2028")</f>
@@ -3951,7 +4100,7 @@
         <f aca="false">Cashflow!N37</f>
         <v>89982</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="23" t="n">
         <f aca="false">D13/$B$4</f>
         <v>0.1499999924985</v>
       </c>
@@ -3959,38 +4108,38 @@
         <f aca="false">SUM($D$9:D13)</f>
         <v>599880.03</v>
       </c>
-      <c r="G13" s="22" t="n">
+      <c r="G13" s="23" t="n">
         <f aca="false">F13/$B$4</f>
         <v>1</v>
       </c>
       <c r="H13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>122</v>
+      <c r="J13" s="2" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D14" s="20" t="n">
         <f aca="false">SUM(D9:D13)</f>
         <v>599880.03</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="24" t="n">
         <f aca="false">D14/B4</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B17" s="5" t="n">
         <f aca="false">ROUND(D14-B4,2)</f>
@@ -4003,10 +4152,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B18" s="5" t="n">
-        <f aca="false">MAX(H9:H12)</f>
+        <f aca="false">MAX(D9:D12)</f>
         <v>239952.01</v>
       </c>
       <c r="C18" s="8" t="str">
@@ -4016,7 +4165,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B19" s="5" t="n">
         <f aca="false">D13</f>
@@ -4029,7 +4178,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B20" s="5" t="n">
         <f aca="false">SUM(D9:D12)</f>
@@ -4037,6 +4186,19 @@
       </c>
       <c r="C20" s="8" t="str">
         <f aca="false">IF(B20&lt;=B4-B6+0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <f aca="false">MIN(I10:I12)</f>
+        <v>0.765999998291325</v>
+      </c>
+      <c r="C21" s="8" t="str">
+        <f aca="false">IF(B21&gt;=Założenia!L5-0.0001,"OK","SPRAWDŹ")</f>
         <v>OK</v>
       </c>
     </row>
@@ -4065,11 +4227,11 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="24" t="str">
+      <c r="A2" s="25" t="str">
         <f aca="false">"Scenariusz wpływu dofinansowania: "&amp;IF(Założenia!B9=1,"1 – zaliczki kwartalne",IF(Założenia!B9=2,"2 – refundacja kwartalna z opóźnieniem "&amp;Założenia!B10&amp;" mies.","3 – wg umowy: zaliczki (max "&amp;TEXT(Założenia!B11,"0%")&amp;") + płatność końcowa "&amp;TEXT(Założenia!B12,"0%")&amp;" po wniosku końcowym"))</f>
         <v>Scenariusz wpływu dofinansowania: 3 – wg umowy: zaliczki (max 40%) + płatność końcowa 15% po wniosku końcowym</v>
       </c>
@@ -4079,95 +4241,95 @@
         <v>29</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="N4" s="16" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="O4" s="16" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B5" s="25" t="n">
+        <v>139</v>
+      </c>
+      <c r="B5" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="25" t="n">
+      <c r="C5" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F5" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="25" t="n">
+      <c r="H5" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="I5" s="25" t="n">
+      <c r="I5" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="25" t="n">
+      <c r="J5" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="K5" s="25" t="n">
+      <c r="K5" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="L5" s="25" t="n">
+      <c r="L5" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="M5" s="25" t="n">
+      <c r="M5" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="N5" s="25" t="n">
+      <c r="N5" s="26" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B6" s="14"/>
       <c r="C6" s="14"/>
@@ -4186,7 +4348,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">SUMPRODUCT((Założenia!$A$22:$A$39=1)*Założenia!D$22:D$39*Założenia!$C$22:$C$39)</f>
@@ -4246,7 +4408,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUMPRODUCT((Założenia!$A$22:$A$39=2)*Założenia!D$22:D$39*Założenia!$C$22:$C$39)</f>
@@ -4306,7 +4468,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">SUMPRODUCT((Założenia!$A$22:$A$39=3)*Założenia!D$22:D$39*Założenia!$C$22:$C$39)</f>
@@ -4366,7 +4528,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B10" s="20" t="n">
         <f aca="false">SUM(B7:B9)</f>
@@ -4416,7 +4578,7 @@
         <f aca="false">SUM(M7:M9)</f>
         <v>44524</v>
       </c>
-      <c r="N10" s="26" t="n">
+      <c r="N10" s="27" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="20" t="n">
@@ -4426,7 +4588,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B11" s="5" t="n">
         <f aca="false">Założenia!$C$15*Założenia!D$15</f>
@@ -4486,7 +4648,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B12" s="5" t="n">
         <f aca="false">Założenia!$C$16*Założenia!D$16</f>
@@ -4546,7 +4708,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B13" s="5" t="n">
         <f aca="false">Założenia!$B$5*B10</f>
@@ -4606,7 +4768,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B14" s="20" t="n">
         <f aca="false">SUM(B10:B13)</f>
@@ -4656,7 +4818,7 @@
         <f aca="false">SUM(M10:M13)</f>
         <v>51202.6</v>
       </c>
-      <c r="N14" s="26" t="n">
+      <c r="N14" s="27" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="20" t="n">
@@ -4666,7 +4828,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B16" s="5" t="n">
         <f aca="false">B10+B13+Założenia!$B$15*Założenia!D$15+Założenia!$B$16*Założenia!D$16</f>
@@ -4726,7 +4888,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B17" s="5" t="n">
         <f aca="false">B14-B16</f>
@@ -4786,7 +4948,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -4805,11 +4967,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,B33,B34,B37)</f>
-        <v>239952.01</v>
+        <v>0</v>
       </c>
       <c r="C20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,C33,C34,C37)</f>
@@ -4817,15 +4979,15 @@
       </c>
       <c r="D20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,D33,D34,D37)</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="E20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,E33,E34,E37)</f>
-        <v>79244.76</v>
+        <v>0</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,F33,F34,F37)</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="G20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,G33,G34,G37)</f>
@@ -4833,11 +4995,11 @@
       </c>
       <c r="H20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,H33,H34,H37)</f>
-        <v>145229.13</v>
+        <v>0</v>
       </c>
       <c r="I20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,I33,I34,I37)</f>
-        <v>0</v>
+        <v>29994.01</v>
       </c>
       <c r="J20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,J33,J34,J37)</f>
@@ -4845,7 +5007,7 @@
       </c>
       <c r="K20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,K33,K34,K37)</f>
-        <v>45472.13</v>
+        <v>0</v>
       </c>
       <c r="L20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,L33,L34,L37)</f>
@@ -4866,53 +5028,53 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B21" s="27" t="n">
+        <v>153</v>
+      </c>
+      <c r="B21" s="28" t="n">
         <f aca="false">Założenia!D17</f>
         <v>0</v>
       </c>
-      <c r="C21" s="27" t="n">
+      <c r="C21" s="28" t="n">
         <f aca="false">Założenia!E17</f>
         <v>0</v>
       </c>
-      <c r="D21" s="27" t="n">
+      <c r="D21" s="28" t="n">
         <f aca="false">Założenia!F17</f>
         <v>0</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E21" s="28" t="n">
         <f aca="false">Założenia!G17</f>
         <v>0</v>
       </c>
-      <c r="F21" s="27" t="n">
+      <c r="F21" s="28" t="n">
         <f aca="false">Założenia!H17</f>
         <v>0</v>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G21" s="28" t="n">
         <f aca="false">Założenia!I17</f>
         <v>0</v>
       </c>
-      <c r="H21" s="27" t="n">
+      <c r="H21" s="28" t="n">
         <f aca="false">Założenia!J17</f>
         <v>0</v>
       </c>
-      <c r="I21" s="27" t="n">
+      <c r="I21" s="28" t="n">
         <f aca="false">Założenia!K17</f>
         <v>0</v>
       </c>
-      <c r="J21" s="27" t="n">
+      <c r="J21" s="28" t="n">
         <f aca="false">Założenia!L17</f>
         <v>0</v>
       </c>
-      <c r="K21" s="27" t="n">
+      <c r="K21" s="28" t="n">
         <f aca="false">Założenia!M17</f>
         <v>0</v>
       </c>
-      <c r="L21" s="27" t="n">
+      <c r="L21" s="28" t="n">
         <f aca="false">Założenia!N17</f>
         <v>0</v>
       </c>
-      <c r="M21" s="27" t="n">
+      <c r="M21" s="28" t="n">
         <f aca="false">Założenia!O17</f>
         <v>0</v>
       </c>
@@ -4926,15 +5088,15 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6,MAX(0,Założenia!$B$8-(B26+B20+B21-B14)))</f>
-        <v>0</v>
+        <v>32802.6</v>
       </c>
       <c r="C22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:B22),MAX(0,Założenia!$B$8-(C26+C20+C21-C14)))</f>
-        <v>0</v>
+        <v>77677.1</v>
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:C22),MAX(0,Założenia!$B$8-(D26+D20+D21-D14)))</f>
@@ -4946,11 +5108,11 @@
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:E22),MAX(0,Założenia!$B$8-(F26+F20+F21-F14)))</f>
-        <v>18261.53</v>
+        <v>0</v>
       </c>
       <c r="G22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:F22),MAX(0,Założenia!$B$8-(G26+G20+G21-G14)))</f>
-        <v>56952.6</v>
+        <v>0</v>
       </c>
       <c r="H22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:G22),MAX(0,Założenia!$B$8-(H26+H20+H21-H14)))</f>
@@ -4962,11 +5124,11 @@
       </c>
       <c r="J22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:I22),MAX(0,Założenia!$B$8-(J26+J20+J21-J14)))</f>
-        <v>25628.67</v>
+        <v>0</v>
       </c>
       <c r="K22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:J22),MAX(0,Założenia!$B$8-(K26+K20+K21-K14)))</f>
-        <v>11480.47</v>
+        <v>1843.57000000002</v>
       </c>
       <c r="L22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:K22),MAX(0,Założenia!$B$8-(L26+L20+L21-L14)))</f>
@@ -4987,47 +5149,47 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>239952.01</v>
+        <v>32802.6</v>
       </c>
       <c r="C23" s="20" t="n">
         <f aca="false">SUM(C20:C22)</f>
-        <v>0</v>
+        <v>77677.1</v>
       </c>
       <c r="D23" s="20" t="n">
         <f aca="false">SUM(D20:D22)</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="E23" s="20" t="n">
         <f aca="false">SUM(E20:E22)</f>
-        <v>79244.76</v>
+        <v>0</v>
       </c>
       <c r="F23" s="20" t="n">
         <f aca="false">SUM(F20:F22)</f>
-        <v>18261.53</v>
+        <v>239952.01</v>
       </c>
       <c r="G23" s="20" t="n">
         <f aca="false">SUM(G20:G22)</f>
-        <v>56952.6</v>
+        <v>0</v>
       </c>
       <c r="H23" s="20" t="n">
         <f aca="false">SUM(H20:H22)</f>
-        <v>145229.13</v>
+        <v>0</v>
       </c>
       <c r="I23" s="20" t="n">
         <f aca="false">SUM(I20:I22)</f>
-        <v>0</v>
+        <v>29994.01</v>
       </c>
       <c r="J23" s="20" t="n">
         <f aca="false">SUM(J20:J22)</f>
-        <v>25628.67</v>
+        <v>0</v>
       </c>
       <c r="K23" s="20" t="n">
         <f aca="false">SUM(K20:K22)</f>
-        <v>56952.6</v>
+        <v>1843.57000000002</v>
       </c>
       <c r="L23" s="20" t="n">
         <f aca="false">SUM(L20:L22)</f>
@@ -5048,7 +5210,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -5067,7 +5229,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B26" s="5" t="n">
         <f aca="false">Założenia!$B$7</f>
@@ -5075,39 +5237,39 @@
       </c>
       <c r="C26" s="5" t="n">
         <f aca="false">B28</f>
-        <v>207149.41</v>
+        <v>0</v>
       </c>
       <c r="D26" s="5" t="n">
         <f aca="false">C28</f>
-        <v>129472.31</v>
+        <v>0</v>
       </c>
       <c r="E26" s="5" t="n">
         <f aca="false">D28</f>
-        <v>27645.21</v>
+        <v>138124.91</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">E28</f>
-        <v>38691.07</v>
+        <v>69926.01</v>
       </c>
       <c r="G26" s="5" t="n">
         <f aca="false">F28</f>
-        <v>0</v>
+        <v>252925.42</v>
       </c>
       <c r="H26" s="5" t="n">
         <f aca="false">G28</f>
-        <v>0</v>
+        <v>195972.82</v>
       </c>
       <c r="I26" s="5" t="n">
         <f aca="false">H28</f>
-        <v>88276.53</v>
+        <v>139020.22</v>
       </c>
       <c r="J26" s="5" t="n">
         <f aca="false">I28</f>
-        <v>31323.93</v>
+        <v>112061.63</v>
       </c>
       <c r="K26" s="5" t="n">
         <f aca="false">J28</f>
-        <v>0</v>
+        <v>55109.03</v>
       </c>
       <c r="L26" s="5" t="n">
         <f aca="false">K28</f>
@@ -5128,47 +5290,47 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B27" s="5" t="n">
         <f aca="false">B23-B14</f>
-        <v>207149.41</v>
+        <v>0</v>
       </c>
       <c r="C27" s="5" t="n">
         <f aca="false">C23-C14</f>
-        <v>-77677.1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="5" t="n">
         <f aca="false">D23-D14</f>
-        <v>-101827.1</v>
+        <v>138124.91</v>
       </c>
       <c r="E27" s="5" t="n">
         <f aca="false">E23-E14</f>
-        <v>11045.86</v>
+        <v>-68198.9</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">F23-F14</f>
-        <v>-38691.07</v>
+        <v>182999.41</v>
       </c>
       <c r="G27" s="5" t="n">
         <f aca="false">G23-G14</f>
-        <v>0</v>
+        <v>-56952.6</v>
       </c>
       <c r="H27" s="5" t="n">
         <f aca="false">H23-H14</f>
-        <v>88276.53</v>
+        <v>-56952.6</v>
       </c>
       <c r="I27" s="5" t="n">
         <f aca="false">I23-I14</f>
-        <v>-56952.6</v>
+        <v>-26958.59</v>
       </c>
       <c r="J27" s="5" t="n">
         <f aca="false">J23-J14</f>
-        <v>-31323.93</v>
+        <v>-56952.6</v>
       </c>
       <c r="K27" s="5" t="n">
         <f aca="false">K23-K14</f>
-        <v>0</v>
+        <v>-55109.03</v>
       </c>
       <c r="L27" s="5" t="n">
         <f aca="false">L23-L14</f>
@@ -5189,43 +5351,43 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B28" s="20" t="n">
         <f aca="false">B26+B27</f>
-        <v>207149.41</v>
+        <v>0</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">C26+C27</f>
-        <v>129472.31</v>
+        <v>0</v>
       </c>
       <c r="D28" s="20" t="n">
         <f aca="false">D26+D27</f>
-        <v>27645.21</v>
+        <v>138124.91</v>
       </c>
       <c r="E28" s="20" t="n">
         <f aca="false">E26+E27</f>
-        <v>38691.07</v>
+        <v>69926.01</v>
       </c>
       <c r="F28" s="20" t="n">
         <f aca="false">F26+F27</f>
-        <v>0</v>
+        <v>252925.42</v>
       </c>
       <c r="G28" s="20" t="n">
         <f aca="false">G26+G27</f>
-        <v>0</v>
+        <v>195972.82</v>
       </c>
       <c r="H28" s="20" t="n">
         <f aca="false">H26+H27</f>
-        <v>88276.53</v>
+        <v>139020.22</v>
       </c>
       <c r="I28" s="20" t="n">
         <f aca="false">I26+I27</f>
-        <v>31323.93</v>
+        <v>112061.63</v>
       </c>
       <c r="J28" s="20" t="n">
         <f aca="false">J26+J27</f>
-        <v>0</v>
+        <v>55109.03</v>
       </c>
       <c r="K28" s="20" t="n">
         <f aca="false">K26+K27</f>
@@ -5250,7 +5412,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-B28)</f>
@@ -5311,43 +5473,43 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B30" s="5" t="n">
         <f aca="false">SUM($B22:B22)</f>
-        <v>0</v>
+        <v>32802.6</v>
       </c>
       <c r="C30" s="5" t="n">
         <f aca="false">SUM($B22:C22)</f>
-        <v>0</v>
+        <v>110479.7</v>
       </c>
       <c r="D30" s="5" t="n">
         <f aca="false">SUM($B22:D22)</f>
-        <v>0</v>
+        <v>110479.7</v>
       </c>
       <c r="E30" s="5" t="n">
         <f aca="false">SUM($B22:E22)</f>
-        <v>0</v>
+        <v>110479.7</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">SUM($B22:F22)</f>
-        <v>18261.53</v>
+        <v>110479.7</v>
       </c>
       <c r="G30" s="5" t="n">
         <f aca="false">SUM($B22:G22)</f>
-        <v>75214.13</v>
+        <v>110479.7</v>
       </c>
       <c r="H30" s="5" t="n">
         <f aca="false">SUM($B22:H22)</f>
-        <v>75214.13</v>
+        <v>110479.7</v>
       </c>
       <c r="I30" s="5" t="n">
         <f aca="false">SUM($B22:I22)</f>
-        <v>75214.13</v>
+        <v>110479.7</v>
       </c>
       <c r="J30" s="5" t="n">
         <f aca="false">SUM($B22:J22)</f>
-        <v>100842.8</v>
+        <v>110479.7</v>
       </c>
       <c r="K30" s="5" t="n">
         <f aca="false">SUM($B22:K22)</f>
@@ -5372,7 +5534,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
@@ -5391,7 +5553,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B33" s="5" t="n">
         <f aca="false">IF(MOD(B$5-1,3)=0,ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;B$5,$B$5:$M$5,"&lt;="&amp;(B$5+2)),2),0)</f>
@@ -5452,7 +5614,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B34" s="5" t="n">
         <f aca="false">IF(AND(B$5-Założenia!$B$10&gt;=3,MOD(B$5-Założenia!$B$10,3)=0),ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;"&amp;(B$5-Założenia!$B$10-3),$B$5:$M$5,"&lt;="&amp;(B$5-Założenia!$B$10)),2),0)</f>
@@ -5513,7 +5675,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B35" s="5" t="n">
         <f aca="false">Założenia!$B$7+B33+B21-B14</f>
@@ -5570,7 +5732,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B36" s="5" t="n">
         <f aca="false">Założenia!$B$7+B34+B21-B14</f>
@@ -5627,54 +5789,54 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B37" s="5" t="n">
-        <f aca="false">MIN(ROUND(Założenia!$B$11*$B$44,2),ROUND((1-Założenia!$B$12)*$B$44,2))</f>
+        <f aca="false">IF(AND(B$5&gt;=Założenia!$L$4,0&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(B$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*0-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-0),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <f aca="false">IF(AND(C$5&gt;=Założenia!$L$4,B41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(C$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*B41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-B41),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <f aca="false">IF(AND(D$5&gt;=Założenia!$L$4,C41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(D$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*C41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-C41),2),0)</f>
         <v>239952.01</v>
       </c>
-      <c r="C37" s="5" t="n">
-        <f aca="false">IF(MOD(C$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-B41,Założenia!$B$11*$B$44-C42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;C$5,$B$5:$M$5,"&lt;="&amp;(C$5+2))-C42)),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <f aca="false">IF(MOD(D$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-C41,Założenia!$B$11*$B$44-D42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;D$5,$B$5:$M$5,"&lt;="&amp;(D$5+2))-D42)),2),0)</f>
-        <v>0</v>
-      </c>
       <c r="E37" s="5" t="n">
-        <f aca="false">IF(MOD(E$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-D41,Założenia!$B$11*$B$44-E42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;E$5,$B$5:$M$5,"&lt;="&amp;(E$5+2))-E42)),2),0)</f>
-        <v>79244.76</v>
+        <f aca="false">IF(AND(E$5&gt;=Założenia!$L$4,D41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(E$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*D41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-D41),2),0)</f>
+        <v>0</v>
       </c>
       <c r="F37" s="5" t="n">
-        <f aca="false">IF(MOD(F$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-E41,Założenia!$B$11*$B$44-F42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;F$5,$B$5:$M$5,"&lt;="&amp;(F$5+2))-F42)),2),0)</f>
-        <v>0</v>
+        <f aca="false">IF(AND(F$5&gt;=Założenia!$L$4,E41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(F$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*E41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-E41),2),0)</f>
+        <v>239952.01</v>
       </c>
       <c r="G37" s="5" t="n">
-        <f aca="false">IF(MOD(G$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-F41,Założenia!$B$11*$B$44-G42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;G$5,$B$5:$M$5,"&lt;="&amp;(G$5+2))-G42)),2),0)</f>
+        <f aca="false">IF(AND(G$5&gt;=Założenia!$L$4,F41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(G$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*F41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-F41),2),0)</f>
         <v>0</v>
       </c>
       <c r="H37" s="5" t="n">
-        <f aca="false">IF(MOD(H$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-G41,Założenia!$B$11*$B$44-H42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;H$5,$B$5:$M$5,"&lt;="&amp;(H$5+2))-H42)),2),0)</f>
-        <v>145229.13</v>
+        <f aca="false">IF(AND(H$5&gt;=Założenia!$L$4,G41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(H$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*G41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-G41),2),0)</f>
+        <v>0</v>
       </c>
       <c r="I37" s="5" t="n">
-        <f aca="false">IF(MOD(I$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-H41,Założenia!$B$11*$B$44-I42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;I$5,$B$5:$M$5,"&lt;="&amp;(I$5+2))-I42)),2),0)</f>
-        <v>0</v>
+        <f aca="false">IF(AND(I$5&gt;=Założenia!$L$4,H41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(I$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*H41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-H41),2),0)</f>
+        <v>29994.01</v>
       </c>
       <c r="J37" s="5" t="n">
-        <f aca="false">IF(MOD(J$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-I41,Założenia!$B$11*$B$44-J42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;J$5,$B$5:$M$5,"&lt;="&amp;(J$5+2))-J42)),2),0)</f>
+        <f aca="false">IF(AND(J$5&gt;=Założenia!$L$4,I41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(J$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*I41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-I41),2),0)</f>
         <v>0</v>
       </c>
       <c r="K37" s="5" t="n">
-        <f aca="false">IF(MOD(K$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-J41,Założenia!$B$11*$B$44-K42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;K$5,$B$5:$M$5,"&lt;="&amp;(K$5+2))-K42)),2),0)</f>
-        <v>45472.13</v>
+        <f aca="false">IF(AND(K$5&gt;=Założenia!$L$4,J41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(K$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*J41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-J41),2),0)</f>
+        <v>0</v>
       </c>
       <c r="L37" s="5" t="n">
-        <f aca="false">IF(MOD(L$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-K41,Założenia!$B$11*$B$44-L42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;L$5,$B$5:$M$5,"&lt;="&amp;(L$5+2))-L42)),2),0)</f>
+        <f aca="false">IF(AND(L$5&gt;=Założenia!$L$4,K41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(L$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*K41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-K41),2),0)</f>
         <v>0</v>
       </c>
       <c r="M37" s="5" t="n">
-        <f aca="false">IF(MOD(M$5-1,3)=0,ROUND(MAX(0,MIN((1-Założenia!$B$12)*$B$44-L41,Założenia!$B$11*$B$44-M42,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;M$5,$B$5:$M$5,"&lt;="&amp;(M$5+2))-M42)),2),0)</f>
+        <f aca="false">IF(AND(M$5&gt;=Założenia!$L$4,L41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(M$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*L41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-L41),2),0)</f>
         <v>0</v>
       </c>
       <c r="N37" s="5" t="n">
@@ -5688,15 +5850,15 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B38" s="5" t="n">
         <f aca="false">Założenia!$B$7+B37+B21-B14</f>
-        <v>207149.41</v>
+        <v>-32802.6</v>
       </c>
       <c r="C38" s="5" t="n">
         <f aca="false">B38+C37+C21-C14</f>
-        <v>129472.31</v>
+        <v>-110479.7</v>
       </c>
       <c r="D38" s="5" t="n">
         <f aca="false">C38+D37+D21-D14</f>
@@ -5704,27 +5866,27 @@
       </c>
       <c r="E38" s="5" t="n">
         <f aca="false">D38+E37+E21-E14</f>
-        <v>38691.07</v>
+        <v>-40553.69</v>
       </c>
       <c r="F38" s="5" t="n">
         <f aca="false">E38+F37+F21-F14</f>
-        <v>-18261.53</v>
+        <v>142445.72</v>
       </c>
       <c r="G38" s="5" t="n">
         <f aca="false">F38+G37+G21-G14</f>
-        <v>-75214.13</v>
+        <v>85493.12</v>
       </c>
       <c r="H38" s="5" t="n">
         <f aca="false">G38+H37+H21-H14</f>
-        <v>13062.4</v>
+        <v>28540.52</v>
       </c>
       <c r="I38" s="5" t="n">
         <f aca="false">H38+I37+I21-I14</f>
-        <v>-43890.2</v>
+        <v>1581.93</v>
       </c>
       <c r="J38" s="5" t="n">
         <f aca="false">I38+J37+J21-J14</f>
-        <v>-100842.8</v>
+        <v>-55370.67</v>
       </c>
       <c r="K38" s="5" t="n">
         <f aca="false">J38+K37+K21-K14</f>
@@ -5745,43 +5907,43 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B39" s="5" t="n">
         <f aca="false">B42+B37</f>
-        <v>239952.01</v>
+        <v>0</v>
       </c>
       <c r="C39" s="5" t="n">
         <f aca="false">C42+C37</f>
-        <v>212069.8</v>
+        <v>0</v>
       </c>
       <c r="D39" s="5" t="n">
         <f aca="false">D42+D37</f>
-        <v>153176.75525</v>
+        <v>239952.01</v>
       </c>
       <c r="E39" s="5" t="n">
         <f aca="false">E42+E37</f>
-        <v>153000.9705</v>
+        <v>73756.2105</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">F42+F37</f>
-        <v>96819.4215</v>
+        <v>257526.6715</v>
       </c>
       <c r="G39" s="5" t="n">
         <f aca="false">G42+G37</f>
-        <v>48409.7115</v>
+        <v>209116.9615</v>
       </c>
       <c r="H39" s="5" t="n">
         <f aca="false">H42+H37</f>
-        <v>145229.1315</v>
+        <v>160707.2515</v>
       </c>
       <c r="I39" s="5" t="n">
         <f aca="false">I42+I37</f>
-        <v>96819.4215000001</v>
+        <v>142291.5515</v>
       </c>
       <c r="J39" s="5" t="n">
         <f aca="false">J42+J37</f>
-        <v>48409.7115000001</v>
+        <v>93881.8415000001</v>
       </c>
       <c r="K39" s="5" t="n">
         <f aca="false">K42+K37</f>
@@ -5801,7 +5963,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B40" s="5" t="n">
         <f aca="false">SUM($B16:B16)</f>
@@ -5858,15 +6020,15 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B41" s="5" t="n">
         <f aca="false">B37</f>
-        <v>239952.01</v>
+        <v>0</v>
       </c>
       <c r="C41" s="5" t="n">
         <f aca="false">B41+C37</f>
-        <v>239952.01</v>
+        <v>0</v>
       </c>
       <c r="D41" s="5" t="n">
         <f aca="false">C41+D37</f>
@@ -5874,27 +6036,27 @@
       </c>
       <c r="E41" s="5" t="n">
         <f aca="false">D41+E37</f>
-        <v>319196.77</v>
+        <v>239952.01</v>
       </c>
       <c r="F41" s="5" t="n">
         <f aca="false">E41+F37</f>
-        <v>319196.77</v>
+        <v>479904.02</v>
       </c>
       <c r="G41" s="5" t="n">
         <f aca="false">F41+G37</f>
-        <v>319196.77</v>
+        <v>479904.02</v>
       </c>
       <c r="H41" s="5" t="n">
         <f aca="false">G41+H37</f>
-        <v>464425.9</v>
+        <v>479904.02</v>
       </c>
       <c r="I41" s="5" t="n">
         <f aca="false">H41+I37</f>
-        <v>464425.9</v>
+        <v>509898.03</v>
       </c>
       <c r="J41" s="5" t="n">
         <f aca="false">I41+J37</f>
-        <v>464425.9</v>
+        <v>509898.03</v>
       </c>
       <c r="K41" s="5" t="n">
         <f aca="false">J41+K37</f>
@@ -5915,18 +6077,18 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B42" s="5" t="n">
         <v>0</v>
       </c>
       <c r="C42" s="5" t="n">
         <f aca="false">MAX(0,B41-Założenia!$B$4*B40)</f>
-        <v>212069.8</v>
+        <v>0</v>
       </c>
       <c r="D42" s="5" t="n">
         <f aca="false">MAX(0,C41-Założenia!$B$4*C40)</f>
-        <v>153176.75525</v>
+        <v>0</v>
       </c>
       <c r="E42" s="5" t="n">
         <f aca="false">MAX(0,D41-Założenia!$B$4*D40)</f>
@@ -5934,27 +6096,27 @@
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">MAX(0,E41-Założenia!$B$4*E40)</f>
-        <v>96819.4215</v>
+        <v>17574.6615</v>
       </c>
       <c r="G42" s="5" t="n">
         <f aca="false">MAX(0,F41-Założenia!$B$4*F40)</f>
-        <v>48409.7115</v>
+        <v>209116.9615</v>
       </c>
       <c r="H42" s="5" t="n">
         <f aca="false">MAX(0,G41-Założenia!$B$4*G40)</f>
-        <v>0.00150000001303852</v>
+        <v>160707.2515</v>
       </c>
       <c r="I42" s="5" t="n">
         <f aca="false">MAX(0,H41-Założenia!$B$4*H40)</f>
-        <v>96819.4215000001</v>
+        <v>112297.5415</v>
       </c>
       <c r="J42" s="5" t="n">
         <f aca="false">MAX(0,I41-Założenia!$B$4*I40)</f>
-        <v>48409.7115000001</v>
+        <v>93881.8415000001</v>
       </c>
       <c r="K42" s="5" t="n">
         <f aca="false">MAX(0,J41-Założenia!$B$4*J40)</f>
-        <v>0.00150000001303852</v>
+        <v>45472.1315</v>
       </c>
       <c r="L42" s="5" t="n">
         <f aca="false">MAX(0,K41-Założenia!$B$4*K40)</f>
@@ -5969,9 +6131,62 @@
         <v>0</v>
       </c>
     </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B43" s="21" t="n">
+        <f aca="false">IF(B37&gt;0,COUNTIF($B37:B37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="21" t="n">
+        <f aca="false">IF(C37&gt;0,COUNTIF($B37:C37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="21" t="n">
+        <f aca="false">IF(D37&gt;0,COUNTIF($B37:D37,"&gt;0"),0)</f>
+        <v>1</v>
+      </c>
+      <c r="E43" s="21" t="n">
+        <f aca="false">IF(E37&gt;0,COUNTIF($B37:E37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="21" t="n">
+        <f aca="false">IF(F37&gt;0,COUNTIF($B37:F37,"&gt;0"),0)</f>
+        <v>2</v>
+      </c>
+      <c r="G43" s="21" t="n">
+        <f aca="false">IF(G37&gt;0,COUNTIF($B37:G37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="21" t="n">
+        <f aca="false">IF(H37&gt;0,COUNTIF($B37:H37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="21" t="n">
+        <f aca="false">IF(I37&gt;0,COUNTIF($B37:I37,"&gt;0"),0)</f>
+        <v>3</v>
+      </c>
+      <c r="J43" s="21" t="n">
+        <f aca="false">IF(J37&gt;0,COUNTIF($B37:J37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K43" s="21" t="n">
+        <f aca="false">IF(K37&gt;0,COUNTIF($B37:K37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L43" s="21" t="n">
+        <f aca="false">IF(L37&gt;0,COUNTIF($B37:L37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M43" s="21" t="n">
+        <f aca="false">IF(M37&gt;0,COUNTIF($B37:M37,"&gt;0"),0)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="B44" s="5" t="n">
         <f aca="false">ROUND(Założenia!$B$4*SUM($B$16:$M$16),2)</f>
@@ -5980,7 +6195,448 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>166</v>
+        <v>175</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3" s="21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D3" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <f aca="false">SUM(Cashflow!B16:D16)</f>
+        <v>195524.47</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <f aca="false">Cashflow!D37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D4" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <f aca="false">Cashflow!E16</f>
+        <v>66095.94</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <f aca="false">Cashflow!E37</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <f aca="false">Cashflow!F16</f>
+        <v>56952.6</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <f aca="false">Cashflow!F37</f>
+        <v>239952.01</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <f aca="false">Cashflow!G16</f>
+        <v>56952.6</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <f aca="false">Cashflow!G37</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <f aca="false">Cashflow!H16</f>
+        <v>56952.6</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <f aca="false">Cashflow!H37</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <f aca="false">Cashflow!I16</f>
+        <v>56952.6</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <f aca="false">Cashflow!I37</f>
+        <v>29994.01</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <f aca="false">Cashflow!J16</f>
+        <v>56952.6</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <f aca="false">Cashflow!J37</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <f aca="false">Cashflow!K16</f>
+        <v>56952.6</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <f aca="false">Cashflow!K37</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <f aca="false">Cashflow!L16</f>
+        <v>51202.6</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <f aca="false">Cashflow!L37</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C12" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D12" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <f aca="false">Cashflow!M16</f>
+        <v>51202.6</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <f aca="false">Cashflow!M37</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <f aca="false">IF(Założenia!$B$10=1,Cashflow!$N$37,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C14" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <f aca="false">IF(Założenia!$B$10=2,Cashflow!$N$37,0)</f>
+        <v>89982</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E15" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F15" s="20" t="n">
+        <f aca="false">SUM(F3:F14)</f>
+        <v>705741.21</v>
+      </c>
+      <c r="G15" s="20" t="n">
+        <f aca="false">SUM(G3:G14)</f>
+        <v>509898.03</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <f aca="false">SUM(H3:H14)</f>
+        <v>89982</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <f aca="false">ROUND(F15-Cashflow!O16,2)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="8" t="str">
+        <f aca="false">IF(ABS(F17)&lt;=0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <f aca="false">ROUND(G15+H15-Cashflow!B44,2)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="8" t="str">
+        <f aca="false">IF(ABS(F18)&lt;=0.05,"OK","SPRAWDŹ")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Przesuń okres projektu na 01.11.2026–31.10.2027, rozliczenia kwartalne wydatków i wniosków o płatność
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Av3yRtjc51k31HhvjViJWB
</commit_message>
<xml_diff>
--- a/Cashflow_SZMO.xlsx
+++ b/Cashflow_SZMO.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="203">
   <si>
     <t xml:space="preserve">Cashflow projektu SZMO – podsumowanie</t>
   </si>
@@ -155,7 +155,7 @@
     <t xml:space="preserve">Założenia modelu cashflow – projekt SZMO (FEPW.01.01-IP.01-0825/26)</t>
   </si>
   <si>
-    <t xml:space="preserve">Smart-ELIT sp. z o.o. · okres realizacji 01.09.2026–31.08.2027 · kolor niebieski = dane wejściowe (z wniosku lub założenie), czarny = formuły</t>
+    <t xml:space="preserve">Smart-ELIT sp. z o.o. · okres realizacji 01.11.2026–31.10.2027 · wnioski o płatność i rozliczenie wydatków co 3 miesiące · kolor niebieski = dane wejściowe (z wniosku lub założenie), czarny = formuły</t>
   </si>
   <si>
     <t xml:space="preserve">Scen. 1: zaliczka na początku kwartału = 85% kosztów kwalif. kolejnych 3 mies. | Scen. 2: refundacja 85% kosztów kwartału z opóźnieniem | Scen. 3: 1. zaliczka = max % z B11, kolejne zaliczki kwartalnie wg potrzeb (niewykorzystana zaliczka ≤ B11, łącznie ≤ 100% − B12), reszta po wniosku końcowym.</t>
@@ -170,7 +170,7 @@
     <t xml:space="preserve">Wniosek – podsumowanie wydatków</t>
   </si>
   <si>
-    <t xml:space="preserve">Miesiąc wypłaty 1. zaliczki (nr mies.: 1 = wrz 2026, 3 = lis 2026)</t>
+    <t xml:space="preserve">Miesiąc wypłaty 1. zaliczki (nr mies.: 1 = lis 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Stawka kosztów pośrednich (od wynagrodzeń kwalifik.)</t>
@@ -188,7 +188,7 @@
     <t xml:space="preserve">Wniosek – źródła finansowania (pożyczka, przedwstępne umowy)</t>
   </si>
   <si>
-    <t xml:space="preserve">Opóźnienie rozliczenia wydatków przed kolejną zaliczką (mies.)</t>
+    <t xml:space="preserve">Opóźnienie: od końca kwartału (wniosek) do wypłaty kolejnej zaliczki (mies.)</t>
   </si>
   <si>
     <t xml:space="preserve">Saldo początkowe gotówki (PLN)</t>
@@ -197,7 +197,7 @@
     <t xml:space="preserve">ZAŁOŻENIE – brak danych we wniosku</t>
   </si>
   <si>
-    <t xml:space="preserve">Wydatkowanie liczone jako 85% × wydatki kwalifikowalne narastająco od początku projektu (w tym wrz–paź 2026).</t>
+    <t xml:space="preserve">Wydatkowanie liczone jako 85% × wydatki kwalifikowalne wykazane we wnioskach o płatność (co 3 mies.: sty, kwi, lip, paź) narastająco od początku projektu.</t>
   </si>
   <si>
     <t xml:space="preserve">Minimalne saldo gotówki / bufor (PLN)</t>
@@ -239,12 +239,6 @@
     <t xml:space="preserve">Brutto (wydatek ogółem)</t>
   </si>
   <si>
-    <t xml:space="preserve">wrz 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">paź 2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">lis 2026</t>
   </si>
   <si>
@@ -275,6 +269,12 @@
     <t xml:space="preserve">sie 2027</t>
   </si>
   <si>
+    <t xml:space="preserve">wrz 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paź 2027</t>
+  </si>
+  <si>
     <t xml:space="preserve">Suma udziałów</t>
   </si>
   <si>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">Przychody ze sprzedaży (wpływ brutto, PLN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Wniosek nie zawiera prognozy przychodów w okresie projektu (pierwsza sprzedaż/pilotaż do 31.08.2027) – domyślnie 0. Terminy płatności zakupów to założenie (zamówienie po rozstrzygnięciu naboru).</t>
+    <t xml:space="preserve">Wniosek nie zawiera prognozy przychodów w okresie projektu (pierwsza sprzedaż/pilotaż do 31.10.2027) – domyślnie 0. Terminy płatności zakupów to założenie (zamówienie po rozstrzygnięciu naboru).</t>
   </si>
   <si>
     <t xml:space="preserve">Zaangażowanie personelu (etaty w miesiącu) i stawki – wg uzasadnień wydatków we wniosku</t>
@@ -413,7 +413,7 @@
     <t xml:space="preserve">Płatność końcowa (refundacja po wniosku o płatność końcową)</t>
   </si>
   <si>
-    <t xml:space="preserve">Wniosek końcowy po 31.08.2027; wypłata poza okresem realizacji projektu</t>
+    <t xml:space="preserve">Wniosek końcowy po 31.10.2027; wypłata poza okresem realizacji projektu</t>
   </si>
   <si>
     <t xml:space="preserve">Kontrola zapisów umowy</t>
@@ -437,7 +437,7 @@
     <t xml:space="preserve">Cashflow projektu SZMO – miesięcznie (PLN)</t>
   </si>
   <si>
-    <t xml:space="preserve">Po projekcie (od wrz 2027)</t>
+    <t xml:space="preserve">Po projekcie (od lis 2027)</t>
   </si>
   <si>
     <t xml:space="preserve">Razem</t>
@@ -551,9 +551,15 @@
     <t xml:space="preserve">Dofinansowanie ogółem (zaokrąglone)</t>
   </si>
   <si>
+    <t xml:space="preserve">Wydatki kwalifikowalne wykazane we wniosku o płatność (co 3 mies.)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pożyczka właścicielska jest uruchamiana automatycznie tylko do poziomu niedoboru gotówki (do limitu z Założeń); spłata pożyczek wspólnikom nie jest w modelu (brak informacji we wniosku). Kolumna „Po projekcie” to wpływy po 31.08.2027 (np. rozliczenie ostatniej transzy).</t>
   </si>
   <si>
+    <t xml:space="preserve">Wydatki kwalifikowalne rozliczane są kwartalnie (wniosek o płatność co 3 mies.: sty, kwi, lip, paź); od nich zależy moment kolejnej zaliczki. Gotówka wydatkowana jest miesięcznie.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dane do Harmonogramu nr 1 (wzór PARP) – wartości z modelu, scenariusz 3</t>
   </si>
   <si>
@@ -626,7 +632,7 @@
     <t xml:space="preserve">Kontrola: zaliczki + refundacja = dofinansowanie</t>
   </si>
   <si>
-    <t xml:space="preserve">Wzór PARP zaczyna się od listopada 2026 – wydatki z wrz–paź 2026 ujęto w wierszu „listopad”. Płatność końcowa w „wrzesień/październik 2027” zależy od Założenia!B10 (1 lub 2). Wartości zostały przeniesione do osobnego pliku według wzoru.</t>
+    <t xml:space="preserve">Wydatki kwalifikowalne wykazano kwartalnie w miesiącu złożenia wniosku o płatność (sty, kwi, lip, paź). Płatność końcowa (refundacja 15%) wpisana w ostatnim wierszu wzoru (paź 2027 = wniosek końcowy); w cashflow wpływa po opóźnieniu z Założenia!B10 (poza okresem projektu).</t>
   </si>
 </sst>
 </file>
@@ -1091,40 +1097,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>wrz 2026</c:v>
+                  <c:v>lis 2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>paź 2026</c:v>
+                  <c:v>gru 2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>lis 2026</c:v>
+                  <c:v>sty 2027</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>gru 2026</c:v>
+                  <c:v>lut 2027</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>sty 2027</c:v>
+                  <c:v>mar 2027</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>lut 2027</c:v>
+                  <c:v>kwi 2027</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>mar 2027</c:v>
+                  <c:v>maj 2027</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>kwi 2027</c:v>
+                  <c:v>cze 2027</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>maj 2027</c:v>
+                  <c:v>lip 2027</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>cze 2027</c:v>
+                  <c:v>sie 2027</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>lip 2027</c:v>
+                  <c:v>wrz 2027</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>sie 2027</c:v>
+                  <c:v>paź 2027</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1142,10 +1148,10 @@
                   <c:v>77677.1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>101827.1</c:v>
+                  <c:v>113073.4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>68198.9</c:v>
+                  <c:v>56952.6</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>56952.6</c:v>
@@ -1229,40 +1235,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>wrz 2026</c:v>
+                  <c:v>lis 2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>paź 2026</c:v>
+                  <c:v>gru 2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>lis 2026</c:v>
+                  <c:v>sty 2027</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>gru 2026</c:v>
+                  <c:v>lut 2027</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>sty 2027</c:v>
+                  <c:v>mar 2027</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>lut 2027</c:v>
+                  <c:v>kwi 2027</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>mar 2027</c:v>
+                  <c:v>maj 2027</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>kwi 2027</c:v>
+                  <c:v>cze 2027</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>maj 2027</c:v>
+                  <c:v>lip 2027</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>cze 2027</c:v>
+                  <c:v>sie 2027</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>lip 2027</c:v>
+                  <c:v>wrz 2027</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>sie 2027</c:v>
+                  <c:v>paź 2027</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1274,16 +1280,16 @@
                 <c:formatCode>#,##0.00;[RED]\(#,##0.00\);\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>32802.6</c:v>
+                  <c:v>239952.01</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>77677.1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>239952.01</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>40553.69</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>239952.01</c:v>
@@ -1295,16 +1301,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>44810.99</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>39381.79</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>29994.01</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1843.57000000002</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>12423.2</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -1315,8 +1321,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="82546140"/>
-        <c:axId val="10554548"/>
+        <c:axId val="71886922"/>
+        <c:axId val="50563773"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -1380,40 +1386,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>wrz 2026</c:v>
+                  <c:v>lis 2026</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>paź 2026</c:v>
+                  <c:v>gru 2026</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>lis 2026</c:v>
+                  <c:v>sty 2027</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>gru 2026</c:v>
+                  <c:v>lut 2027</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>sty 2027</c:v>
+                  <c:v>mar 2027</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>lut 2027</c:v>
+                  <c:v>kwi 2027</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>mar 2027</c:v>
+                  <c:v>maj 2027</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>kwi 2027</c:v>
+                  <c:v>cze 2027</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>maj 2027</c:v>
+                  <c:v>lip 2027</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>cze 2027</c:v>
+                  <c:v>sie 2027</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>lip 2027</c:v>
+                  <c:v>wrz 2027</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>sie 2027</c:v>
+                  <c:v>paź 2027</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1425,34 +1431,34 @@
                 <c:formatCode>#,##0.00;[RED]\(#,##0.00\);\-</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
+                  <c:v>207149.41</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>129472.31</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>16398.91</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="4">
+                  <c:v>182999.41</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>126046.81</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>69094.21</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>12141.61</c:v>
+                </c:pt>
+                <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>138124.91</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>69926.01</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>252925.42</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>195972.82</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>139020.22</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>112061.63</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>55109.03</c:v>
-                </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>-17570.81</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>-38779.4</c:v>
@@ -1473,11 +1479,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="82546140"/>
-        <c:axId val="10554548"/>
+        <c:axId val="71886922"/>
+        <c:axId val="50563773"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="82546140"/>
+        <c:axId val="71886922"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1509,7 +1515,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10554548"/>
+        <c:crossAx val="50563773"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1517,7 +1523,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10554548"/>
+        <c:axId val="50563773"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1559,7 +1565,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82546140"/>
+        <c:crossAx val="71886922"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1991,7 +1997,7 @@
       </c>
       <c r="B16" s="7" t="str">
         <f aca="false">INDEX(Cashflow!B4:M4,MATCH(MIN(Cashflow!B35:M35),Cashflow!B35:M35,0))</f>
-        <v>sie 2027</v>
+        <v>paź 2027</v>
       </c>
       <c r="C16" s="2"/>
     </row>
@@ -2001,7 +2007,7 @@
       </c>
       <c r="B17" s="7" t="str">
         <f aca="false">INDEX(Cashflow!B4:M4,MATCH(MIN(Cashflow!B38:M38),Cashflow!B38:M38,0))</f>
-        <v>sie 2027</v>
+        <v>paź 2027</v>
       </c>
       <c r="C17" s="2"/>
     </row>
@@ -2011,7 +2017,7 @@
       </c>
       <c r="B18" s="7" t="str">
         <f aca="false">INDEX(Cashflow!B4:M4,MATCH(MIN(Cashflow!B36:M36),Cashflow!B36:M36,0))</f>
-        <v>cze 2027</v>
+        <v>sie 2027</v>
       </c>
       <c r="C18" s="2"/>
     </row>
@@ -2276,7 +2282,7 @@
         <v>48</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2310,7 +2316,7 @@
         <v>54</v>
       </c>
       <c r="L6" s="11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2522,10 +2528,10 @@
         <v>0</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" s="10" t="n">
         <v>0</v>
@@ -3977,7 +3983,7 @@
       </c>
       <c r="C10" s="22" t="str">
         <f aca="false">IFERROR(INDEX(Cashflow!$B$4:$M$4,MATCH(2,Cashflow!$B$43:$M$43,0)),"–")</f>
-        <v>sty 2027</v>
+        <v>mar 2027</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">IFERROR(INDEX(Cashflow!$B$37:$M$37,MATCH(2,Cashflow!$B$43:$M$43,0)),0)</f>
@@ -4000,8 +4006,8 @@
         <v>257526.6715</v>
       </c>
       <c r="I10" s="23" t="n">
-        <f aca="false">IFERROR(Założenia!$B$4*INDEX(Cashflow!$B$40:$M$40,MATCH(2,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/F9,"–")</f>
-        <v>0.926757598321431</v>
+        <f aca="false">IFERROR(Założenia!$B$4*SUMIFS(Cashflow!$B$16:$M$16,Cashflow!$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,MATCH(2,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/3)))/F9,"–")</f>
+        <v>0.725010132234358</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>123</v>
@@ -4016,7 +4022,7 @@
       </c>
       <c r="C11" s="22" t="str">
         <f aca="false">IFERROR(INDEX(Cashflow!$B$4:$M$4,MATCH(3,Cashflow!$B$43:$M$43,0)),"–")</f>
-        <v>kwi 2027</v>
+        <v>wrz 2027</v>
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">IFERROR(INDEX(Cashflow!$B$37:$M$37,MATCH(3,Cashflow!$B$43:$M$43,0)),0)</f>
@@ -4036,11 +4042,11 @@
       </c>
       <c r="H11" s="5" t="n">
         <f aca="false">IFERROR(INDEX(Cashflow!$B$39:$M$39,MATCH(3,Cashflow!$B$43:$M$43,0)),0)</f>
-        <v>142291.5515</v>
+        <v>29994.01</v>
       </c>
       <c r="I11" s="23" t="n">
-        <f aca="false">IFERROR(Założenia!$B$4*INDEX(Cashflow!$B$40:$M$40,MATCH(3,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/F10,"–")</f>
-        <v>0.765999998291325</v>
+        <f aca="false">IFERROR(Założenia!$B$4*SUMIFS(Cashflow!$B$16:$M$16,Cashflow!$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,MATCH(3,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/3)))/F10,"–")</f>
+        <v>0.967747464378398</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>125</v>
@@ -4078,7 +4084,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="23" t="str">
-        <f aca="false">IFERROR(Założenia!$B$4*INDEX(Cashflow!$B$40:$M$40,MATCH(4,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/F11,"–")</f>
+        <f aca="false">IFERROR(Założenia!$B$4*SUMIFS(Cashflow!$B$16:$M$16,Cashflow!$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,MATCH(4,Cashflow!$B$43:$M$43,0)-1-Założenia!$L$6)/3)))/F11,"–")</f>
         <v>–</v>
       </c>
       <c r="J12" s="2" t="s">
@@ -4093,8 +4099,8 @@
         <v>128</v>
       </c>
       <c r="C13" s="4" t="str">
-        <f aca="false">CHOOSE(Założenia!B10,"wrz 2027","paź 2027","lis 2027","gru 2027","sty 2028")</f>
-        <v>paź 2027</v>
+        <f aca="false">CHOOSE(Założenia!B10,"lis 2027","gru 2027","sty 2028","lut 2028","mar 2028")</f>
+        <v>gru 2027</v>
       </c>
       <c r="D13" s="5" t="n">
         <f aca="false">Cashflow!N37</f>
@@ -4195,7 +4201,7 @@
       </c>
       <c r="B21" s="5" t="n">
         <f aca="false">MIN(I10:I12)</f>
-        <v>0.765999998291325</v>
+        <v>0.725010132234358</v>
       </c>
       <c r="C21" s="8" t="str">
         <f aca="false">IF(B21&gt;=Założenia!L5-0.0001,"OK","SPRAWDŹ")</f>
@@ -4218,7 +4224,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -4660,11 +4666,11 @@
       </c>
       <c r="D12" s="5" t="n">
         <f aca="false">Założenia!$C$16*Założenia!F$16</f>
-        <v>0</v>
+        <v>11246.3</v>
       </c>
       <c r="E12" s="5" t="n">
         <f aca="false">Założenia!$C$16*Założenia!G$16</f>
-        <v>11246.3</v>
+        <v>0</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">Założenia!$C$16*Założenia!H$16</f>
@@ -4780,11 +4786,11 @@
       </c>
       <c r="D14" s="20" t="n">
         <f aca="false">SUM(D10:D13)</f>
-        <v>101827.1</v>
+        <v>113073.4</v>
       </c>
       <c r="E14" s="20" t="n">
         <f aca="false">SUM(E10:E13)</f>
-        <v>68198.9</v>
+        <v>56952.6</v>
       </c>
       <c r="F14" s="20" t="n">
         <f aca="false">SUM(F10:F13)</f>
@@ -4840,11 +4846,11 @@
       </c>
       <c r="D16" s="5" t="n">
         <f aca="false">D10+D13+Założenia!$B$15*Założenia!F$15+Założenia!$B$16*Założenia!F$16</f>
-        <v>93435.935</v>
+        <v>102579.275</v>
       </c>
       <c r="E16" s="5" t="n">
         <f aca="false">E10+E13+Założenia!$B$15*Założenia!G$15+Założenia!$B$16*Założenia!G$16</f>
-        <v>66095.94</v>
+        <v>56952.6</v>
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">F10+F13+Założenia!$B$15*Założenia!H$15+Założenia!$B$16*Założenia!H$16</f>
@@ -4900,11 +4906,11 @@
       </c>
       <c r="D17" s="5" t="n">
         <f aca="false">D14-D16</f>
-        <v>8391.16500000001</v>
+        <v>10494.125</v>
       </c>
       <c r="E17" s="5" t="n">
         <f aca="false">E14-E16</f>
-        <v>2102.96000000001</v>
+        <v>0</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">F14-F16</f>
@@ -4971,7 +4977,7 @@
       </c>
       <c r="B20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,B33,B34,B37)</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="C20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,C33,C34,C37)</f>
@@ -4979,7 +4985,7 @@
       </c>
       <c r="D20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,D33,D34,D37)</f>
-        <v>239952.01</v>
+        <v>0</v>
       </c>
       <c r="E20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,E33,E34,E37)</f>
@@ -4999,7 +5005,7 @@
       </c>
       <c r="I20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,I33,I34,I37)</f>
-        <v>29994.01</v>
+        <v>0</v>
       </c>
       <c r="J20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,J33,J34,J37)</f>
@@ -5011,7 +5017,7 @@
       </c>
       <c r="L20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,L33,L34,L37)</f>
-        <v>0</v>
+        <v>29994.01</v>
       </c>
       <c r="M20" s="5" t="n">
         <f aca="false">CHOOSE(Założenia!$B$9,M33,M34,M37)</f>
@@ -5092,11 +5098,11 @@
       </c>
       <c r="B22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6,MAX(0,Założenia!$B$8-(B26+B20+B21-B14)))</f>
-        <v>32802.6</v>
+        <v>0</v>
       </c>
       <c r="C22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:B22),MAX(0,Założenia!$B$8-(C26+C20+C21-C14)))</f>
-        <v>77677.1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:C22),MAX(0,Założenia!$B$8-(D26+D20+D21-D14)))</f>
@@ -5104,7 +5110,7 @@
       </c>
       <c r="E22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:D22),MAX(0,Założenia!$B$8-(E26+E20+E21-E14)))</f>
-        <v>0</v>
+        <v>40553.69</v>
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:E22),MAX(0,Założenia!$B$8-(F26+F20+F21-F14)))</f>
@@ -5124,15 +5130,15 @@
       </c>
       <c r="J22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:I22),MAX(0,Założenia!$B$8-(J26+J20+J21-J14)))</f>
-        <v>0</v>
+        <v>44810.99</v>
       </c>
       <c r="K22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:J22),MAX(0,Założenia!$B$8-(K26+K20+K21-K14)))</f>
-        <v>1843.57000000002</v>
+        <v>39381.79</v>
       </c>
       <c r="L22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:K22),MAX(0,Założenia!$B$8-(L26+L20+L21-L14)))</f>
-        <v>12423.2</v>
+        <v>0</v>
       </c>
       <c r="M22" s="5" t="n">
         <f aca="false">MIN(Założenia!$B$6-SUM($B22:L22),MAX(0,Założenia!$B$8-(M26+M20+M21-M14)))</f>
@@ -5153,19 +5159,19 @@
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">SUM(B20:B22)</f>
-        <v>32802.6</v>
+        <v>239952.01</v>
       </c>
       <c r="C23" s="20" t="n">
         <f aca="false">SUM(C20:C22)</f>
-        <v>77677.1</v>
+        <v>0</v>
       </c>
       <c r="D23" s="20" t="n">
         <f aca="false">SUM(D20:D22)</f>
-        <v>239952.01</v>
+        <v>0</v>
       </c>
       <c r="E23" s="20" t="n">
         <f aca="false">SUM(E20:E22)</f>
-        <v>0</v>
+        <v>40553.69</v>
       </c>
       <c r="F23" s="20" t="n">
         <f aca="false">SUM(F20:F22)</f>
@@ -5181,19 +5187,19 @@
       </c>
       <c r="I23" s="20" t="n">
         <f aca="false">SUM(I20:I22)</f>
-        <v>29994.01</v>
+        <v>0</v>
       </c>
       <c r="J23" s="20" t="n">
         <f aca="false">SUM(J20:J22)</f>
-        <v>0</v>
+        <v>44810.99</v>
       </c>
       <c r="K23" s="20" t="n">
         <f aca="false">SUM(K20:K22)</f>
-        <v>1843.57000000002</v>
+        <v>39381.79</v>
       </c>
       <c r="L23" s="20" t="n">
         <f aca="false">SUM(L20:L22)</f>
-        <v>12423.2</v>
+        <v>29994.01</v>
       </c>
       <c r="M23" s="20" t="n">
         <f aca="false">SUM(M20:M22)</f>
@@ -5237,43 +5243,43 @@
       </c>
       <c r="C26" s="5" t="n">
         <f aca="false">B28</f>
-        <v>0</v>
+        <v>207149.41</v>
       </c>
       <c r="D26" s="5" t="n">
         <f aca="false">C28</f>
-        <v>0</v>
+        <v>129472.31</v>
       </c>
       <c r="E26" s="5" t="n">
         <f aca="false">D28</f>
-        <v>138124.91</v>
+        <v>16398.91</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">E28</f>
-        <v>69926.01</v>
+        <v>0</v>
       </c>
       <c r="G26" s="5" t="n">
         <f aca="false">F28</f>
-        <v>252925.42</v>
+        <v>182999.41</v>
       </c>
       <c r="H26" s="5" t="n">
         <f aca="false">G28</f>
-        <v>195972.82</v>
+        <v>126046.81</v>
       </c>
       <c r="I26" s="5" t="n">
         <f aca="false">H28</f>
-        <v>139020.22</v>
+        <v>69094.21</v>
       </c>
       <c r="J26" s="5" t="n">
         <f aca="false">I28</f>
-        <v>112061.63</v>
+        <v>12141.61</v>
       </c>
       <c r="K26" s="5" t="n">
         <f aca="false">J28</f>
-        <v>55109.03</v>
+        <v>0</v>
       </c>
       <c r="L26" s="5" t="n">
         <f aca="false">K28</f>
-        <v>0</v>
+        <v>-17570.81</v>
       </c>
       <c r="M26" s="5" t="n">
         <f aca="false">L28</f>
@@ -5294,19 +5300,19 @@
       </c>
       <c r="B27" s="5" t="n">
         <f aca="false">B23-B14</f>
-        <v>0</v>
+        <v>207149.41</v>
       </c>
       <c r="C27" s="5" t="n">
         <f aca="false">C23-C14</f>
-        <v>0</v>
+        <v>-77677.1</v>
       </c>
       <c r="D27" s="5" t="n">
         <f aca="false">D23-D14</f>
-        <v>138124.91</v>
+        <v>-113073.4</v>
       </c>
       <c r="E27" s="5" t="n">
         <f aca="false">E23-E14</f>
-        <v>-68198.9</v>
+        <v>-16398.91</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">F23-F14</f>
@@ -5322,19 +5328,19 @@
       </c>
       <c r="I27" s="5" t="n">
         <f aca="false">I23-I14</f>
-        <v>-26958.59</v>
+        <v>-56952.6</v>
       </c>
       <c r="J27" s="5" t="n">
         <f aca="false">J23-J14</f>
-        <v>-56952.6</v>
+        <v>-12141.61</v>
       </c>
       <c r="K27" s="5" t="n">
         <f aca="false">K23-K14</f>
-        <v>-55109.03</v>
+        <v>-17570.81</v>
       </c>
       <c r="L27" s="5" t="n">
         <f aca="false">L23-L14</f>
-        <v>-38779.4</v>
+        <v>-21208.59</v>
       </c>
       <c r="M27" s="5" t="n">
         <f aca="false">M23-M14</f>
@@ -5355,43 +5361,43 @@
       </c>
       <c r="B28" s="20" t="n">
         <f aca="false">B26+B27</f>
-        <v>0</v>
+        <v>207149.41</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">C26+C27</f>
-        <v>0</v>
+        <v>129472.31</v>
       </c>
       <c r="D28" s="20" t="n">
         <f aca="false">D26+D27</f>
-        <v>138124.91</v>
+        <v>16398.91</v>
       </c>
       <c r="E28" s="20" t="n">
         <f aca="false">E26+E27</f>
-        <v>69926.01</v>
+        <v>0</v>
       </c>
       <c r="F28" s="20" t="n">
         <f aca="false">F26+F27</f>
-        <v>252925.42</v>
+        <v>182999.41</v>
       </c>
       <c r="G28" s="20" t="n">
         <f aca="false">G26+G27</f>
-        <v>195972.82</v>
+        <v>126046.81</v>
       </c>
       <c r="H28" s="20" t="n">
         <f aca="false">H26+H27</f>
-        <v>139020.22</v>
+        <v>69094.21</v>
       </c>
       <c r="I28" s="20" t="n">
         <f aca="false">I26+I27</f>
-        <v>112061.63</v>
+        <v>12141.61</v>
       </c>
       <c r="J28" s="20" t="n">
         <f aca="false">J26+J27</f>
-        <v>55109.03</v>
+        <v>0</v>
       </c>
       <c r="K28" s="20" t="n">
         <f aca="false">K26+K27</f>
-        <v>0</v>
+        <v>-17570.81</v>
       </c>
       <c r="L28" s="20" t="n">
         <f aca="false">L26+L27</f>
@@ -5452,7 +5458,7 @@
       </c>
       <c r="K29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-K28)</f>
-        <v>0</v>
+        <v>17570.81</v>
       </c>
       <c r="L29" s="5" t="n">
         <f aca="false">MAX(0,Założenia!$B$8-L28)</f>
@@ -5477,43 +5483,43 @@
       </c>
       <c r="B30" s="5" t="n">
         <f aca="false">SUM($B22:B22)</f>
-        <v>32802.6</v>
+        <v>0</v>
       </c>
       <c r="C30" s="5" t="n">
         <f aca="false">SUM($B22:C22)</f>
-        <v>110479.7</v>
+        <v>0</v>
       </c>
       <c r="D30" s="5" t="n">
         <f aca="false">SUM($B22:D22)</f>
-        <v>110479.7</v>
+        <v>0</v>
       </c>
       <c r="E30" s="5" t="n">
         <f aca="false">SUM($B22:E22)</f>
-        <v>110479.7</v>
+        <v>40553.69</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">SUM($B22:F22)</f>
-        <v>110479.7</v>
+        <v>40553.69</v>
       </c>
       <c r="G30" s="5" t="n">
         <f aca="false">SUM($B22:G22)</f>
-        <v>110479.7</v>
+        <v>40553.69</v>
       </c>
       <c r="H30" s="5" t="n">
         <f aca="false">SUM($B22:H22)</f>
-        <v>110479.7</v>
+        <v>40553.69</v>
       </c>
       <c r="I30" s="5" t="n">
         <f aca="false">SUM($B22:I22)</f>
-        <v>110479.7</v>
+        <v>40553.69</v>
       </c>
       <c r="J30" s="5" t="n">
         <f aca="false">SUM($B22:J22)</f>
-        <v>110479.7</v>
+        <v>85364.68</v>
       </c>
       <c r="K30" s="5" t="n">
         <f aca="false">SUM($B22:K22)</f>
-        <v>112323.27</v>
+        <v>124746.47</v>
       </c>
       <c r="L30" s="5" t="n">
         <f aca="false">SUM($B22:L22)</f>
@@ -5557,7 +5563,7 @@
       </c>
       <c r="B33" s="5" t="n">
         <f aca="false">IF(MOD(B$5-1,3)=0,ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;B$5,$B$5:$M$5,"&lt;="&amp;(B$5+2)),2),0)</f>
-        <v>166195.8</v>
+        <v>173967.64</v>
       </c>
       <c r="C33" s="5" t="n">
         <f aca="false">IF(MOD(C$5-1,3)=0,ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;C$5,$B$5:$M$5,"&lt;="&amp;(C$5+2)),2),0)</f>
@@ -5569,7 +5575,7 @@
       </c>
       <c r="E33" s="5" t="n">
         <f aca="false">IF(MOD(E$5-1,3)=0,ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;E$5,$B$5:$M$5,"&lt;="&amp;(E$5+2)),2),0)</f>
-        <v>153000.97</v>
+        <v>145229.13</v>
       </c>
       <c r="F33" s="5" t="n">
         <f aca="false">IF(MOD(F$5-1,3)=0,ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;="&amp;F$5,$B$5:$M$5,"&lt;="&amp;(F$5+2)),2),0)</f>
@@ -5634,7 +5640,7 @@
       </c>
       <c r="F34" s="5" t="n">
         <f aca="false">IF(AND(F$5-Założenia!$B$10&gt;=3,MOD(F$5-Założenia!$B$10,3)=0),ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;"&amp;(F$5-Założenia!$B$10-3),$B$5:$M$5,"&lt;="&amp;(F$5-Założenia!$B$10)),2),0)</f>
-        <v>166195.8</v>
+        <v>173967.64</v>
       </c>
       <c r="G34" s="5" t="n">
         <f aca="false">IF(AND(G$5-Założenia!$B$10&gt;=3,MOD(G$5-Założenia!$B$10,3)=0),ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;"&amp;(G$5-Założenia!$B$10-3),$B$5:$M$5,"&lt;="&amp;(G$5-Założenia!$B$10)),2),0)</f>
@@ -5646,7 +5652,7 @@
       </c>
       <c r="I34" s="5" t="n">
         <f aca="false">IF(AND(I$5-Założenia!$B$10&gt;=3,MOD(I$5-Założenia!$B$10,3)=0),ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;"&amp;(I$5-Założenia!$B$10-3),$B$5:$M$5,"&lt;="&amp;(I$5-Założenia!$B$10)),2),0)</f>
-        <v>153000.97</v>
+        <v>145229.13</v>
       </c>
       <c r="J34" s="5" t="n">
         <f aca="false">IF(AND(J$5-Założenia!$B$10&gt;=3,MOD(J$5-Założenia!$B$10,3)=0),ROUND(Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&gt;"&amp;(J$5-Założenia!$B$10-3),$B$5:$M$5,"&lt;="&amp;(J$5-Założenia!$B$10)),2),0)</f>
@@ -5679,15 +5685,15 @@
       </c>
       <c r="B35" s="5" t="n">
         <f aca="false">Założenia!$B$7+B33+B21-B14</f>
-        <v>133393.2</v>
+        <v>141165.04</v>
       </c>
       <c r="C35" s="5" t="n">
         <f aca="false">B35+C33+C21-C14</f>
-        <v>55716.1</v>
+        <v>63487.94</v>
       </c>
       <c r="D35" s="5" t="n">
         <f aca="false">C35+D33+D21-D14</f>
-        <v>-46111</v>
+        <v>-49585.46</v>
       </c>
       <c r="E35" s="5" t="n">
         <f aca="false">D35+E33+E21-E14</f>
@@ -5744,7 +5750,7 @@
       </c>
       <c r="D36" s="5" t="n">
         <f aca="false">C36+D34+D21-D14</f>
-        <v>-212306.8</v>
+        <v>-223553.1</v>
       </c>
       <c r="E36" s="5" t="n">
         <f aca="false">D36+E34+E21-E14</f>
@@ -5752,15 +5758,15 @@
       </c>
       <c r="F36" s="5" t="n">
         <f aca="false">E36+F34+F21-F14</f>
-        <v>-171262.5</v>
+        <v>-163490.66</v>
       </c>
       <c r="G36" s="5" t="n">
         <f aca="false">F36+G34+G21-G14</f>
-        <v>-228215.1</v>
+        <v>-220443.26</v>
       </c>
       <c r="H36" s="5" t="n">
         <f aca="false">G36+H34+H21-H14</f>
-        <v>-285167.7</v>
+        <v>-277395.86</v>
       </c>
       <c r="I36" s="5" t="n">
         <f aca="false">H36+I34+I21-I14</f>
@@ -5792,51 +5798,51 @@
         <v>167</v>
       </c>
       <c r="B37" s="5" t="n">
-        <f aca="false">IF(AND(B$5&gt;=Założenia!$L$4,0&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(B$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*0-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-0),2),0)</f>
-        <v>0</v>
+        <f aca="false">IF(AND(B$5&gt;=Założenia!$L$4,0&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,B$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*0-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-0),2),0)</f>
+        <v>239952.01</v>
       </c>
       <c r="C37" s="5" t="n">
-        <f aca="false">IF(AND(C$5&gt;=Założenia!$L$4,B41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(C$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*B41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-B41),2),0)</f>
+        <f aca="false">IF(AND(C$5&gt;=Założenia!$L$4,B41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,C$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*B41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-B41),2),0)</f>
         <v>0</v>
       </c>
       <c r="D37" s="5" t="n">
-        <f aca="false">IF(AND(D$5&gt;=Założenia!$L$4,C41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(D$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*C41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-C41),2),0)</f>
+        <f aca="false">IF(AND(D$5&gt;=Założenia!$L$4,C41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,D$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*C41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-C41),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <f aca="false">IF(AND(E$5&gt;=Założenia!$L$4,D41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,E$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*D41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-D41),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <f aca="false">IF(AND(F$5&gt;=Założenia!$L$4,E41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,F$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*E41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-E41),2),0)</f>
         <v>239952.01</v>
       </c>
-      <c r="E37" s="5" t="n">
-        <f aca="false">IF(AND(E$5&gt;=Założenia!$L$4,D41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(E$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*D41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-D41),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="F37" s="5" t="n">
-        <f aca="false">IF(AND(F$5&gt;=Założenia!$L$4,E41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(F$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*E41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-E41),2),0)</f>
-        <v>239952.01</v>
-      </c>
       <c r="G37" s="5" t="n">
-        <f aca="false">IF(AND(G$5&gt;=Założenia!$L$4,F41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(G$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*F41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-F41),2),0)</f>
+        <f aca="false">IF(AND(G$5&gt;=Założenia!$L$4,F41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,G$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*F41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-F41),2),0)</f>
         <v>0</v>
       </c>
       <c r="H37" s="5" t="n">
-        <f aca="false">IF(AND(H$5&gt;=Założenia!$L$4,G41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(H$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*G41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-G41),2),0)</f>
+        <f aca="false">IF(AND(H$5&gt;=Założenia!$L$4,G41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,H$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*G41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-G41),2),0)</f>
         <v>0</v>
       </c>
       <c r="I37" s="5" t="n">
-        <f aca="false">IF(AND(I$5&gt;=Założenia!$L$4,H41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(I$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*H41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-H41),2),0)</f>
+        <f aca="false">IF(AND(I$5&gt;=Założenia!$L$4,H41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,I$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*H41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-H41),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <f aca="false">IF(AND(J$5&gt;=Założenia!$L$4,I41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,J$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*I41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-I41),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <f aca="false">IF(AND(K$5&gt;=Założenia!$L$4,J41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,K$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*J41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-J41),2),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L37" s="5" t="n">
+        <f aca="false">IF(AND(L$5&gt;=Założenia!$L$4,K41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,L$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*K41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-K41),2),0)</f>
         <v>29994.01</v>
       </c>
-      <c r="J37" s="5" t="n">
-        <f aca="false">IF(AND(J$5&gt;=Założenia!$L$4,I41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(J$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*I41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-I41),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="K37" s="5" t="n">
-        <f aca="false">IF(AND(K$5&gt;=Założenia!$L$4,J41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(K$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*J41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-J41),2),0)</f>
-        <v>0</v>
-      </c>
-      <c r="L37" s="5" t="n">
-        <f aca="false">IF(AND(L$5&gt;=Założenia!$L$4,K41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(L$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*K41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-K41),2),0)</f>
-        <v>0</v>
-      </c>
       <c r="M37" s="5" t="n">
-        <f aca="false">IF(AND(M$5&gt;=Założenia!$L$4,L41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(M$5-1-Założenia!$L$6))&gt;=Założenia!$L$5*L41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-L41),2),0)</f>
+        <f aca="false">IF(AND(M$5&gt;=Założenia!$L$4,L41&lt;(1-Założenia!$B$12)*$B$44-0.005,Założenia!$B$4*SUMIFS($B$16:$M$16,$B$5:$M$5,"&lt;="&amp;(3*INT(MAX(0,M$5-1-Założenia!$L$6)/3)))&gt;=Założenia!$L$5*L41-0.005),ROUND(MIN(Założenia!$B$11*$B$44,(1-Założenia!$B$12)*$B$44-L41),2),0)</f>
         <v>0</v>
       </c>
       <c r="N37" s="5" t="n">
@@ -5854,15 +5860,15 @@
       </c>
       <c r="B38" s="5" t="n">
         <f aca="false">Założenia!$B$7+B37+B21-B14</f>
-        <v>-32802.6</v>
+        <v>207149.41</v>
       </c>
       <c r="C38" s="5" t="n">
         <f aca="false">B38+C37+C21-C14</f>
-        <v>-110479.7</v>
+        <v>129472.31</v>
       </c>
       <c r="D38" s="5" t="n">
         <f aca="false">C38+D37+D21-D14</f>
-        <v>27645.21</v>
+        <v>16398.91</v>
       </c>
       <c r="E38" s="5" t="n">
         <f aca="false">D38+E37+E21-E14</f>
@@ -5882,15 +5888,15 @@
       </c>
       <c r="I38" s="5" t="n">
         <f aca="false">H38+I37+I21-I14</f>
-        <v>1581.93</v>
+        <v>-28412.08</v>
       </c>
       <c r="J38" s="5" t="n">
         <f aca="false">I38+J37+J21-J14</f>
-        <v>-55370.67</v>
+        <v>-85364.68</v>
       </c>
       <c r="K38" s="5" t="n">
         <f aca="false">J38+K37+K21-K14</f>
-        <v>-112323.27</v>
+        <v>-142317.28</v>
       </c>
       <c r="L38" s="5" t="n">
         <f aca="false">K38+L37+L21-L14</f>
@@ -5911,19 +5917,19 @@
       </c>
       <c r="B39" s="5" t="n">
         <f aca="false">B42+B37</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="C39" s="5" t="n">
         <f aca="false">C42+C37</f>
-        <v>0</v>
+        <v>212069.8</v>
       </c>
       <c r="D39" s="5" t="n">
         <f aca="false">D42+D37</f>
-        <v>239952.01</v>
+        <v>153176.75525</v>
       </c>
       <c r="E39" s="5" t="n">
         <f aca="false">E42+E37</f>
-        <v>73756.2105</v>
+        <v>65984.3715</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">F42+F37</f>
@@ -5939,19 +5945,19 @@
       </c>
       <c r="I39" s="5" t="n">
         <f aca="false">I42+I37</f>
-        <v>142291.5515</v>
+        <v>112297.5415</v>
       </c>
       <c r="J39" s="5" t="n">
         <f aca="false">J42+J37</f>
-        <v>93881.8415000001</v>
+        <v>63887.8315000001</v>
       </c>
       <c r="K39" s="5" t="n">
         <f aca="false">K42+K37</f>
-        <v>45472.1315</v>
+        <v>15478.1215</v>
       </c>
       <c r="L39" s="5" t="n">
         <f aca="false">L42+L37</f>
-        <v>0</v>
+        <v>29994.01</v>
       </c>
       <c r="M39" s="5" t="n">
         <f aca="false">M42+M37</f>
@@ -5975,7 +5981,7 @@
       </c>
       <c r="D40" s="5" t="n">
         <f aca="false">SUM($B16:D16)</f>
-        <v>195524.47</v>
+        <v>204667.81</v>
       </c>
       <c r="E40" s="5" t="n">
         <f aca="false">SUM($B16:E16)</f>
@@ -6024,11 +6030,11 @@
       </c>
       <c r="B41" s="5" t="n">
         <f aca="false">B37</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="C41" s="5" t="n">
         <f aca="false">B41+C37</f>
-        <v>0</v>
+        <v>239952.01</v>
       </c>
       <c r="D41" s="5" t="n">
         <f aca="false">C41+D37</f>
@@ -6052,15 +6058,15 @@
       </c>
       <c r="I41" s="5" t="n">
         <f aca="false">H41+I37</f>
-        <v>509898.03</v>
+        <v>479904.02</v>
       </c>
       <c r="J41" s="5" t="n">
         <f aca="false">I41+J37</f>
-        <v>509898.03</v>
+        <v>479904.02</v>
       </c>
       <c r="K41" s="5" t="n">
         <f aca="false">J41+K37</f>
-        <v>509898.03</v>
+        <v>479904.02</v>
       </c>
       <c r="L41" s="5" t="n">
         <f aca="false">K41+L37</f>
@@ -6084,15 +6090,15 @@
       </c>
       <c r="C42" s="5" t="n">
         <f aca="false">MAX(0,B41-Założenia!$B$4*B40)</f>
-        <v>0</v>
+        <v>212069.8</v>
       </c>
       <c r="D42" s="5" t="n">
         <f aca="false">MAX(0,C41-Założenia!$B$4*C40)</f>
-        <v>0</v>
+        <v>153176.75525</v>
       </c>
       <c r="E42" s="5" t="n">
         <f aca="false">MAX(0,D41-Założenia!$B$4*D40)</f>
-        <v>73756.2105</v>
+        <v>65984.3715</v>
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">MAX(0,E41-Założenia!$B$4*E40)</f>
@@ -6112,11 +6118,11 @@
       </c>
       <c r="J42" s="5" t="n">
         <f aca="false">MAX(0,I41-Założenia!$B$4*I40)</f>
-        <v>93881.8415000001</v>
+        <v>63887.8315000001</v>
       </c>
       <c r="K42" s="5" t="n">
         <f aca="false">MAX(0,J41-Założenia!$B$4*J40)</f>
-        <v>45472.1315</v>
+        <v>15478.1215</v>
       </c>
       <c r="L42" s="5" t="n">
         <f aca="false">MAX(0,K41-Założenia!$B$4*K40)</f>
@@ -6137,7 +6143,7 @@
       </c>
       <c r="B43" s="21" t="n">
         <f aca="false">IF(B37&gt;0,COUNTIF($B37:B37,"&gt;0"),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" s="21" t="n">
         <f aca="false">IF(C37&gt;0,COUNTIF($B37:C37,"&gt;0"),0)</f>
@@ -6145,7 +6151,7 @@
       </c>
       <c r="D43" s="21" t="n">
         <f aca="false">IF(D37&gt;0,COUNTIF($B37:D37,"&gt;0"),0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" s="21" t="n">
         <f aca="false">IF(E37&gt;0,COUNTIF($B37:E37,"&gt;0"),0)</f>
@@ -6165,7 +6171,7 @@
       </c>
       <c r="I43" s="21" t="n">
         <f aca="false">IF(I37&gt;0,COUNTIF($B37:I37,"&gt;0"),0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J43" s="21" t="n">
         <f aca="false">IF(J37&gt;0,COUNTIF($B37:J37,"&gt;0"),0)</f>
@@ -6177,7 +6183,7 @@
       </c>
       <c r="L43" s="21" t="n">
         <f aca="false">IF(L37&gt;0,COUNTIF($B37:L37,"&gt;0"),0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M43" s="21" t="n">
         <f aca="false">IF(M37&gt;0,COUNTIF($B37:M37,"&gt;0"),0)</f>
@@ -6193,9 +6199,66 @@
         <v>599880.03</v>
       </c>
     </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <f aca="false">SUM(B16:D16)</f>
+        <v>204667.81</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <f aca="false">SUM(E16:G16)</f>
+        <v>170857.8</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="5" t="n">
+        <f aca="false">SUM(H16:J16)</f>
+        <v>170857.8</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="5" t="n">
+        <f aca="false">SUM(K16:M16)</f>
+        <v>159357.8</v>
+      </c>
+      <c r="N45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="20" t="n">
+        <f aca="false">SUM(B45:N45)</f>
+        <v>705741.21</v>
+      </c>
+    </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2" t="s">
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -6228,41 +6291,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E2" s="15" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F2" s="15" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C3" s="21" t="n">
         <v>2026</v>
@@ -6271,14 +6334,14 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F3" s="5" t="n">
-        <f aca="false">SUM(Cashflow!B16:D16)</f>
-        <v>195524.47</v>
+        <f aca="false">Cashflow!B45</f>
+        <v>0</v>
       </c>
       <c r="G3" s="5" t="n">
-        <f aca="false">Cashflow!D37</f>
+        <f aca="false">Cashflow!B37</f>
         <v>239952.01</v>
       </c>
       <c r="H3" s="5" t="n">
@@ -6287,10 +6350,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C4" s="21" t="n">
         <v>2026</v>
@@ -6299,14 +6362,14 @@
         <v>4</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F4" s="5" t="n">
-        <f aca="false">Cashflow!E16</f>
-        <v>66095.94</v>
+        <f aca="false">Cashflow!C45</f>
+        <v>0</v>
       </c>
       <c r="G4" s="5" t="n">
-        <f aca="false">Cashflow!E37</f>
+        <f aca="false">Cashflow!C37</f>
         <v>0</v>
       </c>
       <c r="H4" s="5" t="n">
@@ -6315,10 +6378,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C5" s="21" t="n">
         <v>2027</v>
@@ -6327,82 +6390,82 @@
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F5" s="5" t="n">
-        <f aca="false">Cashflow!F16</f>
-        <v>56952.6</v>
+        <f aca="false">Cashflow!D45</f>
+        <v>204667.81</v>
       </c>
       <c r="G5" s="5" t="n">
+        <f aca="false">Cashflow!D37</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <f aca="false">Cashflow!E45</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <f aca="false">Cashflow!E37</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <f aca="false">Cashflow!F45</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="n">
         <f aca="false">Cashflow!F37</f>
         <v>239952.01</v>
       </c>
-      <c r="H5" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C6" s="21" t="n">
-        <v>2027</v>
-      </c>
-      <c r="D6" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <f aca="false">Cashflow!G16</f>
-        <v>56952.6</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <f aca="false">Cashflow!G37</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C7" s="21" t="n">
-        <v>2027</v>
-      </c>
-      <c r="D7" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <f aca="false">Cashflow!H16</f>
-        <v>56952.6</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <f aca="false">Cashflow!H37</f>
-        <v>0</v>
-      </c>
       <c r="H7" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C8" s="21" t="n">
         <v>2027</v>
@@ -6411,15 +6474,15 @@
         <v>2</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F8" s="5" t="n">
-        <f aca="false">Cashflow!I16</f>
-        <v>56952.6</v>
+        <f aca="false">Cashflow!G45</f>
+        <v>170857.8</v>
       </c>
       <c r="G8" s="5" t="n">
-        <f aca="false">Cashflow!I37</f>
-        <v>29994.01</v>
+        <f aca="false">Cashflow!G37</f>
+        <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
         <v>0</v>
@@ -6427,10 +6490,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C9" s="21" t="n">
         <v>2027</v>
@@ -6439,14 +6502,14 @@
         <v>2</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F9" s="5" t="n">
-        <f aca="false">Cashflow!J16</f>
-        <v>56952.6</v>
+        <f aca="false">Cashflow!H45</f>
+        <v>0</v>
       </c>
       <c r="G9" s="5" t="n">
-        <f aca="false">Cashflow!J37</f>
+        <f aca="false">Cashflow!H37</f>
         <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
@@ -6455,10 +6518,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C10" s="21" t="n">
         <v>2027</v>
@@ -6467,14 +6530,14 @@
         <v>2</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F10" s="5" t="n">
-        <f aca="false">Cashflow!K16</f>
-        <v>56952.6</v>
+        <f aca="false">Cashflow!I45</f>
+        <v>0</v>
       </c>
       <c r="G10" s="5" t="n">
-        <f aca="false">Cashflow!K37</f>
+        <f aca="false">Cashflow!I37</f>
         <v>0</v>
       </c>
       <c r="H10" s="5" t="n">
@@ -6483,10 +6546,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C11" s="21" t="n">
         <v>2027</v>
@@ -6495,14 +6558,14 @@
         <v>3</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F11" s="5" t="n">
-        <f aca="false">Cashflow!L16</f>
-        <v>51202.6</v>
+        <f aca="false">Cashflow!J45</f>
+        <v>170857.8</v>
       </c>
       <c r="G11" s="5" t="n">
-        <f aca="false">Cashflow!L37</f>
+        <f aca="false">Cashflow!J37</f>
         <v>0</v>
       </c>
       <c r="H11" s="5" t="n">
@@ -6511,10 +6574,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C12" s="21" t="n">
         <v>2027</v>
@@ -6523,14 +6586,14 @@
         <v>3</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F12" s="5" t="n">
-        <f aca="false">Cashflow!M16</f>
-        <v>51202.6</v>
+        <f aca="false">Cashflow!K45</f>
+        <v>0</v>
       </c>
       <c r="G12" s="5" t="n">
-        <f aca="false">Cashflow!M37</f>
+        <f aca="false">Cashflow!K37</f>
         <v>0</v>
       </c>
       <c r="H12" s="5" t="n">
@@ -6539,10 +6602,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C13" s="21" t="n">
         <v>2027</v>
@@ -6551,25 +6614,26 @@
         <v>3</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F13" s="5" t="n">
+        <f aca="false">Cashflow!L45</f>
         <v>0</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0</v>
+        <f aca="false">Cashflow!L37</f>
+        <v>29994.01</v>
       </c>
       <c r="H13" s="5" t="n">
-        <f aca="false">IF(Założenia!$B$10=1,Cashflow!$N$37,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C14" s="21" t="n">
         <v>2027</v>
@@ -6578,16 +6642,18 @@
         <v>4</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <f aca="false">Cashflow!M45</f>
+        <v>159357.8</v>
       </c>
       <c r="G14" s="5" t="n">
+        <f aca="false">Cashflow!M37</f>
         <v>0</v>
       </c>
       <c r="H14" s="5" t="n">
-        <f aca="false">IF(Założenia!$B$10=2,Cashflow!$N$37,0)</f>
+        <f aca="false">Cashflow!$N$37</f>
         <v>89982</v>
       </c>
     </row>
@@ -6610,7 +6676,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">ROUND(F15-Cashflow!O16,2)</f>
@@ -6623,7 +6689,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F18" s="5" t="n">
         <f aca="false">ROUND(G15+H15-Cashflow!B44,2)</f>
@@ -6636,7 +6702,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>